<commit_message>
Atualiza planilha de disponibilidade - 08/10/2026 11:16
</commit_message>
<xml_diff>
--- a/disponibilidade.xlsx
+++ b/disponibilidade.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rafael.germano\Documents\Rafael Germano\Codex\2026-05-19\app disponiblidade\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE9C81CD-F619-4710-B189-E0DBDA203255}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94497724-9416-4A22-BD98-382E2A2D7F9C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="743" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="823" uniqueCount="74">
   <si>
     <t>Modelo de Disponibilidade por Cultura e Packing</t>
   </si>
@@ -247,6 +247,9 @@
   </si>
   <si>
     <t>Extrinha</t>
+  </si>
+  <si>
+    <t>CEAGESP</t>
   </si>
 </sst>
 </file>
@@ -362,7 +365,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -425,7 +428,6 @@
     <xf numFmtId="3" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -440,6 +442,23 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -615,16 +634,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="20.25" customHeight="1">
-      <c r="A1" s="24" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
+      <c r="A1" s="30" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
     </row>
     <row r="3" spans="1:8" ht="29.25" customHeight="1">
       <c r="A3" s="1" t="s">
@@ -692,7 +711,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:N91"/>
+  <dimension ref="A1:N133"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="22.25" style="11" customWidth="1"/>
@@ -767,39 +786,41 @@
       </c>
       <c r="B5" s="21">
         <f>SUM(B6:B7)</f>
-        <v>0</v>
+        <v>2700</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>20</v>
       </c>
       <c r="G5" s="14">
         <f>SUM(G6:G7)</f>
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="K5" s="7" t="s">
         <v>20</v>
       </c>
       <c r="L5" s="14">
         <f>SUM(L6:L7)</f>
-        <v>2300</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="15" customHeight="1">
       <c r="A6" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="14"/>
+      <c r="B6" s="14">
+        <v>2700</v>
+      </c>
       <c r="F6" s="7" t="s">
         <v>21</v>
       </c>
       <c r="G6" s="14">
-        <v>200</v>
+        <v>400</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>21</v>
       </c>
       <c r="L6" s="14">
-        <v>2300</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="15" customHeight="1">
@@ -822,7 +843,7 @@
       </c>
       <c r="B8" s="15">
         <f>SUM(B9:B10)</f>
-        <v>0</v>
+        <v>340</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>23</v>
@@ -836,14 +857,16 @@
       </c>
       <c r="L8" s="15">
         <f>SUM(L9:L10)</f>
-        <v>700</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="15" customHeight="1">
       <c r="A9" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="15"/>
+      <c r="B9" s="15">
+        <v>340</v>
+      </c>
       <c r="F9" s="9" t="s">
         <v>21</v>
       </c>
@@ -852,7 +875,7 @@
         <v>21</v>
       </c>
       <c r="L9" s="15">
-        <v>700</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="15" customHeight="1">
@@ -933,14 +956,14 @@
       </c>
       <c r="G14" s="15">
         <f>SUM(G15:G16)</f>
-        <v>0</v>
+        <v>130</v>
       </c>
       <c r="K14" s="9" t="s">
         <v>25</v>
       </c>
       <c r="L14" s="15">
         <f>SUM(L15:L16)</f>
-        <v>170</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="15" customHeight="1">
@@ -951,13 +974,13 @@
       <c r="F15" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="G15" s="15"/>
+      <c r="G15" s="15">
+        <v>130</v>
+      </c>
       <c r="K15" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="L15" s="15">
-        <v>170</v>
-      </c>
+      <c r="L15" s="15"/>
     </row>
     <row r="16" spans="1:14" ht="15" customHeight="1">
       <c r="A16" s="9" t="s">
@@ -979,7 +1002,7 @@
       </c>
       <c r="B17" s="14">
         <f>SUM(B18:B19)</f>
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F17" s="7" t="s">
         <v>26</v>
@@ -1000,7 +1023,9 @@
       <c r="A18" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B18" s="14"/>
+      <c r="B18" s="14">
+        <v>50</v>
+      </c>
       <c r="F18" s="7" t="s">
         <v>21</v>
       </c>
@@ -1030,7 +1055,7 @@
       </c>
       <c r="B20" s="15">
         <f>SUM(B21:B22)</f>
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="F20" s="9" t="s">
         <v>27</v>
@@ -1051,7 +1076,9 @@
       <c r="A21" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="B21" s="15"/>
+      <c r="B21" s="15">
+        <v>300</v>
+      </c>
       <c r="F21" s="9" t="s">
         <v>21</v>
       </c>
@@ -1139,7 +1166,7 @@
       </c>
       <c r="G26" s="15">
         <f>SUM(G27:G28)</f>
-        <v>500</v>
+        <v>157</v>
       </c>
       <c r="K26" s="9" t="s">
         <v>29</v>
@@ -1158,7 +1185,7 @@
         <v>21</v>
       </c>
       <c r="G27" s="15">
-        <v>500</v>
+        <v>157</v>
       </c>
       <c r="K27" s="9" t="s">
         <v>21</v>
@@ -1199,7 +1226,7 @@
       </c>
       <c r="L29" s="14">
         <f>SUM(L30:L31)</f>
-        <v>750</v>
+        <v>720</v>
       </c>
     </row>
     <row r="30" spans="1:12" ht="15" customHeight="1">
@@ -1215,7 +1242,7 @@
         <v>21</v>
       </c>
       <c r="L30" s="14">
-        <v>750</v>
+        <v>720</v>
       </c>
     </row>
     <row r="31" spans="1:12" ht="15" customHeight="1">
@@ -1252,7 +1279,7 @@
       </c>
       <c r="L32" s="15">
         <f>SUM(L33:L34)</f>
-        <v>63</v>
+        <v>190</v>
       </c>
     </row>
     <row r="33" spans="1:14" ht="15" customHeight="1">
@@ -1268,7 +1295,7 @@
         <v>21</v>
       </c>
       <c r="L33" s="15">
-        <v>63</v>
+        <v>190</v>
       </c>
     </row>
     <row r="34" spans="1:14" ht="15" customHeight="1">
@@ -1356,7 +1383,7 @@
       </c>
       <c r="L38" s="23">
         <f>SUM(L39:L40)</f>
-        <v>17</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:14" ht="15" customHeight="1">
@@ -1371,9 +1398,7 @@
       <c r="K39" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="L39" s="15">
-        <v>17</v>
-      </c>
+      <c r="L39" s="15"/>
     </row>
     <row r="40" spans="1:14" ht="15" customHeight="1">
       <c r="A40" s="9" t="s">
@@ -1395,21 +1420,21 @@
       </c>
       <c r="B41" s="13">
         <f>SUM(B5,B8,B11,B14,B17,B20,B23,B26,B29,B32,B35,B38)</f>
-        <v>0</v>
+        <v>3390</v>
       </c>
       <c r="F41" s="8" t="s">
         <v>34</v>
       </c>
       <c r="G41" s="13">
         <f>SUM(G5,G8,G11,G14,G17,G20,G23,G26,G29,G32,G35,G38)</f>
-        <v>700</v>
+        <v>687</v>
       </c>
       <c r="K41" s="8" t="s">
         <v>34</v>
       </c>
       <c r="L41" s="13">
         <f>SUM(L5,L8,L11,L14,L17,L20,L23,L26,L29,L32,L35,L38)</f>
-        <v>4000</v>
+        <v>6010</v>
       </c>
     </row>
     <row r="42" spans="1:14" ht="15" customHeight="1">
@@ -1505,7 +1530,7 @@
       </c>
       <c r="B53" s="14">
         <f>SUM(B54:B55)</f>
-        <v>750</v>
+        <v>0</v>
       </c>
       <c r="F53" s="7" t="s">
         <v>20</v>
@@ -1519,16 +1544,14 @@
       </c>
       <c r="L53" s="14">
         <f>SUM(L54:L55)</f>
-        <v>2700</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="54" spans="1:14" ht="15" customHeight="1">
       <c r="A54" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B54" s="14">
-        <v>750</v>
-      </c>
+      <c r="B54" s="14"/>
       <c r="F54" s="7" t="s">
         <v>21</v>
       </c>
@@ -1537,7 +1560,7 @@
         <v>21</v>
       </c>
       <c r="L54" s="14">
-        <v>2700</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="55" spans="1:14" ht="15" customHeight="1">
@@ -1662,7 +1685,7 @@
       </c>
       <c r="B62" s="15">
         <f>SUM(B63:B64)</f>
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F62" s="9" t="s">
         <v>25</v>
@@ -1676,7 +1699,7 @@
       </c>
       <c r="L62" s="15">
         <f>SUM(L63:L64)</f>
-        <v>350</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63" spans="1:14" ht="15" customHeight="1">
@@ -1684,7 +1707,7 @@
         <v>21</v>
       </c>
       <c r="B63" s="15">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F63" s="9" t="s">
         <v>21</v>
@@ -1693,9 +1716,7 @@
       <c r="K63" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="L63" s="15">
-        <v>350</v>
-      </c>
+      <c r="L63" s="15"/>
     </row>
     <row r="64" spans="1:14" ht="15" customHeight="1">
       <c r="A64" s="9" t="s">
@@ -2127,7 +2148,7 @@
       </c>
       <c r="B89" s="13">
         <f>SUM(B53,B56,B59,B62,B65,B68,B71,B74,B77,B80,B83,B86)</f>
-        <v>820</v>
+        <v>60</v>
       </c>
       <c r="F89" s="8" t="s">
         <v>34</v>
@@ -2141,7 +2162,7 @@
       </c>
       <c r="L89" s="13">
         <f>SUM(L53,L56,L59,L62,L65,L68,L71,L74,L77,L80,L83,L86)</f>
-        <v>3050</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="90" spans="1:14" ht="15" customHeight="1">
@@ -2171,6 +2192,628 @@
       <c r="L91" s="9"/>
       <c r="M91" s="9"/>
       <c r="N91" s="9"/>
+    </row>
+    <row r="93" spans="1:14" ht="15">
+      <c r="A93" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="B93" s="24"/>
+      <c r="C93" s="24"/>
+      <c r="D93" s="24"/>
+      <c r="E93" s="24"/>
+      <c r="F93" s="29" t="s">
+        <v>15</v>
+      </c>
+      <c r="G93" s="24"/>
+    </row>
+    <row r="94" spans="1:14" ht="15">
+      <c r="A94" s="10">
+        <f>A46</f>
+        <v>0</v>
+      </c>
+      <c r="B94" s="24"/>
+      <c r="C94" s="24"/>
+      <c r="D94" s="24"/>
+      <c r="E94" s="24"/>
+      <c r="F94" s="10">
+        <f>F46</f>
+        <v>0</v>
+      </c>
+      <c r="G94" s="24"/>
+    </row>
+    <row r="95" spans="1:14" ht="15">
+      <c r="A95" s="9"/>
+      <c r="B95" s="9"/>
+      <c r="C95" s="9"/>
+      <c r="D95" s="9"/>
+      <c r="E95" s="24"/>
+      <c r="F95" s="9"/>
+      <c r="G95" s="9"/>
+    </row>
+    <row r="96" spans="1:14" ht="15">
+      <c r="A96" s="27" t="s">
+        <v>73</v>
+      </c>
+      <c r="B96" s="24"/>
+      <c r="C96" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="D96" s="24"/>
+      <c r="E96" s="24"/>
+      <c r="F96" s="27" t="s">
+        <v>73</v>
+      </c>
+      <c r="G96" s="24"/>
+      <c r="H96" s="27" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" ht="15">
+      <c r="A97" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B97" s="26">
+        <f>SUM(B98:B99)</f>
+        <v>946</v>
+      </c>
+      <c r="C97" s="24"/>
+      <c r="D97" s="24"/>
+      <c r="E97" s="24"/>
+      <c r="F97" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="G97" s="26">
+        <f>SUM(G98:G99)</f>
+        <v>633</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" ht="15">
+      <c r="A98" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B98" s="26">
+        <v>946</v>
+      </c>
+      <c r="C98" s="24"/>
+      <c r="D98" s="24"/>
+      <c r="E98" s="24"/>
+      <c r="F98" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G98" s="26">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" ht="15">
+      <c r="A99" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B99" s="26"/>
+      <c r="C99" s="24"/>
+      <c r="D99" s="24"/>
+      <c r="E99" s="24"/>
+      <c r="F99" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G99" s="26"/>
+    </row>
+    <row r="100" spans="1:7" ht="15">
+      <c r="A100" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B100" s="25">
+        <f>SUM(B101:B102)</f>
+        <v>0</v>
+      </c>
+      <c r="C100" s="24"/>
+      <c r="D100" s="24"/>
+      <c r="E100" s="24"/>
+      <c r="F100" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="G100" s="25">
+        <f>SUM(G101:G102)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" ht="15">
+      <c r="A101" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B101" s="25"/>
+      <c r="C101" s="24"/>
+      <c r="D101" s="24"/>
+      <c r="E101" s="24"/>
+      <c r="F101" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G101" s="25"/>
+    </row>
+    <row r="102" spans="1:7" ht="15">
+      <c r="A102" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B102" s="25"/>
+      <c r="C102" s="24"/>
+      <c r="D102" s="24"/>
+      <c r="E102" s="24"/>
+      <c r="F102" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G102" s="25"/>
+    </row>
+    <row r="103" spans="1:7" ht="15">
+      <c r="A103" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B103" s="26">
+        <f>SUM(B104:B105)</f>
+        <v>0</v>
+      </c>
+      <c r="C103" s="24"/>
+      <c r="D103" s="24"/>
+      <c r="E103" s="24"/>
+      <c r="F103" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="G103" s="26">
+        <f>SUM(G104:G105)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" ht="15">
+      <c r="A104" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B104" s="26"/>
+      <c r="C104" s="24"/>
+      <c r="D104" s="24"/>
+      <c r="E104" s="24"/>
+      <c r="F104" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G104" s="26"/>
+    </row>
+    <row r="105" spans="1:7" ht="15">
+      <c r="A105" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B105" s="26"/>
+      <c r="C105" s="24"/>
+      <c r="D105" s="24"/>
+      <c r="E105" s="24"/>
+      <c r="F105" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G105" s="26"/>
+    </row>
+    <row r="106" spans="1:7" ht="15">
+      <c r="A106" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B106" s="25">
+        <f>SUM(B107:B108)</f>
+        <v>0</v>
+      </c>
+      <c r="C106" s="24"/>
+      <c r="D106" s="24"/>
+      <c r="E106" s="24"/>
+      <c r="F106" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="G106" s="25">
+        <f>SUM(G107:G108)</f>
+        <v>374</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" ht="15">
+      <c r="A107" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B107" s="25"/>
+      <c r="C107" s="24"/>
+      <c r="D107" s="24"/>
+      <c r="E107" s="24"/>
+      <c r="F107" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G107" s="25">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" ht="15">
+      <c r="A108" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B108" s="25"/>
+      <c r="C108" s="24"/>
+      <c r="D108" s="24"/>
+      <c r="E108" s="24"/>
+      <c r="F108" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G108" s="25"/>
+    </row>
+    <row r="109" spans="1:7" ht="15">
+      <c r="A109" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B109" s="26">
+        <f>SUM(B110:B111)</f>
+        <v>0</v>
+      </c>
+      <c r="C109" s="24"/>
+      <c r="D109" s="24"/>
+      <c r="E109" s="24"/>
+      <c r="F109" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G109" s="26">
+        <f>SUM(G110:G111)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" ht="15">
+      <c r="A110" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B110" s="26"/>
+      <c r="C110" s="24"/>
+      <c r="D110" s="24"/>
+      <c r="E110" s="24"/>
+      <c r="F110" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G110" s="26"/>
+    </row>
+    <row r="111" spans="1:7" ht="15">
+      <c r="A111" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B111" s="26"/>
+      <c r="C111" s="24"/>
+      <c r="D111" s="24"/>
+      <c r="E111" s="24"/>
+      <c r="F111" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G111" s="26"/>
+    </row>
+    <row r="112" spans="1:7" ht="15">
+      <c r="A112" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B112" s="25">
+        <f>SUM(B113:B114)</f>
+        <v>0</v>
+      </c>
+      <c r="C112" s="24"/>
+      <c r="D112" s="24"/>
+      <c r="E112" s="24"/>
+      <c r="F112" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="G112" s="25">
+        <f>SUM(G113:G114)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" ht="15">
+      <c r="A113" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B113" s="25"/>
+      <c r="C113" s="24"/>
+      <c r="D113" s="24"/>
+      <c r="E113" s="24"/>
+      <c r="F113" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G113" s="25"/>
+    </row>
+    <row r="114" spans="1:7" ht="15">
+      <c r="A114" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B114" s="25"/>
+      <c r="C114" s="24"/>
+      <c r="D114" s="24"/>
+      <c r="E114" s="24"/>
+      <c r="F114" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G114" s="25"/>
+    </row>
+    <row r="115" spans="1:7" ht="15">
+      <c r="A115" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="B115" s="26">
+        <f>SUM(B116:B117)</f>
+        <v>0</v>
+      </c>
+      <c r="C115" s="24"/>
+      <c r="D115" s="24"/>
+      <c r="E115" s="24"/>
+      <c r="F115" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="G115" s="26">
+        <f>SUM(G116:G117)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" ht="15">
+      <c r="A116" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B116" s="26"/>
+      <c r="C116" s="24"/>
+      <c r="D116" s="24"/>
+      <c r="E116" s="24"/>
+      <c r="F116" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G116" s="26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" ht="15">
+      <c r="A117" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B117" s="26"/>
+      <c r="C117" s="24"/>
+      <c r="D117" s="24"/>
+      <c r="E117" s="24"/>
+      <c r="F117" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G117" s="26"/>
+    </row>
+    <row r="118" spans="1:7" ht="15">
+      <c r="A118" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="B118" s="25">
+        <f>SUM(B119:B120)</f>
+        <v>0</v>
+      </c>
+      <c r="C118" s="24"/>
+      <c r="D118" s="24"/>
+      <c r="E118" s="24"/>
+      <c r="F118" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="G118" s="25">
+        <f>SUM(G119:G120)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" ht="15">
+      <c r="A119" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B119" s="25"/>
+      <c r="C119" s="24"/>
+      <c r="D119" s="24"/>
+      <c r="E119" s="24"/>
+      <c r="F119" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G119" s="25"/>
+    </row>
+    <row r="120" spans="1:7" ht="15">
+      <c r="A120" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B120" s="25"/>
+      <c r="C120" s="24"/>
+      <c r="D120" s="24"/>
+      <c r="E120" s="24"/>
+      <c r="F120" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G120" s="25"/>
+    </row>
+    <row r="121" spans="1:7" ht="15">
+      <c r="A121" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B121" s="26">
+        <f>SUM(B122:B123)</f>
+        <v>0</v>
+      </c>
+      <c r="C121" s="24"/>
+      <c r="D121" s="24"/>
+      <c r="E121" s="24"/>
+      <c r="F121" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="G121" s="26">
+        <f>SUM(G122:G123)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" ht="15">
+      <c r="A122" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B122" s="26"/>
+      <c r="C122" s="24"/>
+      <c r="D122" s="24"/>
+      <c r="E122" s="24"/>
+      <c r="F122" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G122" s="26"/>
+    </row>
+    <row r="123" spans="1:7" ht="15">
+      <c r="A123" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B123" s="26"/>
+      <c r="C123" s="24"/>
+      <c r="D123" s="24"/>
+      <c r="E123" s="24"/>
+      <c r="F123" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G123" s="26"/>
+    </row>
+    <row r="124" spans="1:7" ht="15">
+      <c r="A124" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B124" s="25">
+        <f>SUM(B125:B126)</f>
+        <v>0</v>
+      </c>
+      <c r="C124" s="24"/>
+      <c r="D124" s="24"/>
+      <c r="E124" s="24"/>
+      <c r="F124" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="G124" s="25">
+        <f>SUM(G125:G126)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" ht="15">
+      <c r="A125" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B125" s="25"/>
+      <c r="C125" s="24"/>
+      <c r="D125" s="24"/>
+      <c r="E125" s="24"/>
+      <c r="F125" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G125" s="25"/>
+    </row>
+    <row r="126" spans="1:7" ht="15">
+      <c r="A126" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B126" s="25"/>
+      <c r="C126" s="24"/>
+      <c r="D126" s="24"/>
+      <c r="E126" s="24"/>
+      <c r="F126" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G126" s="25"/>
+    </row>
+    <row r="127" spans="1:7" ht="15">
+      <c r="A127" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="B127" s="26">
+        <f>SUM(B128:B129)</f>
+        <v>0</v>
+      </c>
+      <c r="C127" s="24"/>
+      <c r="D127" s="24"/>
+      <c r="E127" s="24"/>
+      <c r="F127" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="G127" s="26">
+        <f>SUM(G128:G129)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7" ht="15">
+      <c r="A128" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B128" s="26"/>
+      <c r="C128" s="24"/>
+      <c r="D128" s="24"/>
+      <c r="E128" s="24"/>
+      <c r="F128" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G128" s="26"/>
+    </row>
+    <row r="129" spans="1:7" ht="15">
+      <c r="A129" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B129" s="26"/>
+      <c r="C129" s="24"/>
+      <c r="D129" s="24"/>
+      <c r="E129" s="24"/>
+      <c r="F129" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G129" s="26"/>
+    </row>
+    <row r="130" spans="1:7" ht="15">
+      <c r="A130" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="B130" s="25">
+        <f>SUM(B131:B132)</f>
+        <v>0</v>
+      </c>
+      <c r="C130" s="24"/>
+      <c r="D130" s="24"/>
+      <c r="E130" s="24"/>
+      <c r="F130" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="G130" s="25">
+        <f>SUM(G131:G132)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" ht="15">
+      <c r="A131" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B131" s="25"/>
+      <c r="C131" s="24"/>
+      <c r="D131" s="24"/>
+      <c r="E131" s="24"/>
+      <c r="F131" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="G131" s="25"/>
+    </row>
+    <row r="132" spans="1:7" ht="15">
+      <c r="A132" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B132" s="25"/>
+      <c r="C132" s="24"/>
+      <c r="D132" s="24"/>
+      <c r="E132" s="24"/>
+      <c r="F132" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="G132" s="25"/>
+    </row>
+    <row r="133" spans="1:7" ht="15">
+      <c r="A133" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="B133" s="28">
+        <f>SUM(B97,B100,B103,B106,B109,B112,B115,B118,B121,B124,B127,B130)</f>
+        <v>946</v>
+      </c>
+      <c r="C133" s="24"/>
+      <c r="D133" s="24"/>
+      <c r="E133" s="24"/>
+      <c r="F133" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="G133" s="28">
+        <f>SUM(G97,G100,G103,G106,G109,G112,G115,G118,G121,G124,G127,G130)</f>
+        <v>1007</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2191,44 +2834,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15" customHeight="1">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="F1" s="30" t="s">
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="F1" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="K1" s="30" t="s">
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="K1" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="L1" s="25"/>
-      <c r="M1" s="25"/>
-      <c r="N1" s="25"/>
+      <c r="L1" s="31"/>
+      <c r="M1" s="31"/>
+      <c r="N1" s="31"/>
     </row>
     <row r="2" spans="1:14" ht="15" customHeight="1">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="F2" s="30" t="s">
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="F2" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="K2" s="30" t="s">
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="K2" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="L2" s="25"/>
-      <c r="M2" s="25"/>
-      <c r="N2" s="25"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="31"/>
     </row>
     <row r="3" spans="1:14" ht="15" customHeight="1">
       <c r="A3" s="9"/>
@@ -2245,191 +2888,191 @@
       <c r="N3" s="9"/>
     </row>
     <row r="4" spans="1:14" ht="15" customHeight="1">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="25"/>
-      <c r="C4" s="28" t="s">
+      <c r="B4" s="31"/>
+      <c r="C4" s="35" t="s">
         <v>38</v>
       </c>
-      <c r="D4" s="25"/>
-      <c r="F4" s="28" t="s">
+      <c r="D4" s="31"/>
+      <c r="F4" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="G4" s="25"/>
-      <c r="H4" s="28" t="s">
+      <c r="G4" s="31"/>
+      <c r="H4" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="I4" s="25"/>
-      <c r="K4" s="28" t="s">
+      <c r="I4" s="31"/>
+      <c r="K4" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="L4" s="25"/>
-      <c r="M4" s="28" t="s">
+      <c r="L4" s="31"/>
+      <c r="M4" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="N4" s="25"/>
+      <c r="N4" s="31"/>
     </row>
     <row r="5" spans="1:14" ht="15" customHeight="1">
       <c r="A5" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="27">
+      <c r="B5" s="34">
         <v>352</v>
       </c>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="31"/>
       <c r="F5" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G5" s="27"/>
-      <c r="H5" s="25"/>
-      <c r="I5" s="25"/>
+      <c r="G5" s="34"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="31"/>
       <c r="K5" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="L5" s="27"/>
-      <c r="M5" s="25"/>
-      <c r="N5" s="25"/>
+      <c r="L5" s="34"/>
+      <c r="M5" s="31"/>
+      <c r="N5" s="31"/>
     </row>
     <row r="6" spans="1:14" ht="15" customHeight="1">
       <c r="A6" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="26">
+      <c r="B6" s="33">
         <v>376</v>
       </c>
-      <c r="C6" s="25"/>
-      <c r="D6" s="25"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="31"/>
       <c r="F6" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="G6" s="26"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="25"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="31"/>
+      <c r="I6" s="31"/>
       <c r="K6" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="L6" s="26"/>
-      <c r="M6" s="25"/>
-      <c r="N6" s="25"/>
+      <c r="L6" s="33"/>
+      <c r="M6" s="31"/>
+      <c r="N6" s="31"/>
     </row>
     <row r="7" spans="1:14" ht="15" customHeight="1">
       <c r="A7" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="27">
-        <v>0</v>
-      </c>
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
+      <c r="B7" s="34">
+        <v>0</v>
+      </c>
+      <c r="C7" s="31"/>
+      <c r="D7" s="31"/>
       <c r="F7" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G7" s="27"/>
-      <c r="H7" s="25"/>
-      <c r="I7" s="25"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="31"/>
+      <c r="I7" s="31"/>
       <c r="K7" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="L7" s="27"/>
-      <c r="M7" s="25"/>
-      <c r="N7" s="25"/>
+      <c r="L7" s="34"/>
+      <c r="M7" s="31"/>
+      <c r="N7" s="31"/>
     </row>
     <row r="8" spans="1:14" ht="15" customHeight="1">
       <c r="A8" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="26">
+      <c r="B8" s="33">
         <v>724</v>
       </c>
-      <c r="C8" s="25"/>
-      <c r="D8" s="25"/>
+      <c r="C8" s="31"/>
+      <c r="D8" s="31"/>
       <c r="F8" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="G8" s="26"/>
-      <c r="H8" s="25"/>
-      <c r="I8" s="25"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="31"/>
+      <c r="I8" s="31"/>
       <c r="K8" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="L8" s="26"/>
-      <c r="M8" s="25"/>
-      <c r="N8" s="25"/>
+      <c r="L8" s="33"/>
+      <c r="M8" s="31"/>
+      <c r="N8" s="31"/>
     </row>
     <row r="9" spans="1:14" ht="15" customHeight="1">
       <c r="A9" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B9" s="27">
+      <c r="B9" s="34">
         <v>411</v>
       </c>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
+      <c r="C9" s="31"/>
+      <c r="D9" s="31"/>
       <c r="F9" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G9" s="27"/>
-      <c r="H9" s="25"/>
-      <c r="I9" s="25"/>
+      <c r="G9" s="34"/>
+      <c r="H9" s="31"/>
+      <c r="I9" s="31"/>
       <c r="K9" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="L9" s="27"/>
-      <c r="M9" s="25"/>
-      <c r="N9" s="25"/>
+      <c r="L9" s="34"/>
+      <c r="M9" s="31"/>
+      <c r="N9" s="31"/>
     </row>
     <row r="10" spans="1:14" ht="15" customHeight="1">
       <c r="A10" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="B10" s="26">
-        <v>0</v>
-      </c>
-      <c r="C10" s="25"/>
-      <c r="D10" s="25"/>
+      <c r="B10" s="33">
+        <v>0</v>
+      </c>
+      <c r="C10" s="31"/>
+      <c r="D10" s="31"/>
       <c r="F10" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="G10" s="26"/>
-      <c r="H10" s="25"/>
-      <c r="I10" s="25"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="31"/>
       <c r="K10" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="L10" s="26"/>
-      <c r="M10" s="25"/>
-      <c r="N10" s="25"/>
+      <c r="L10" s="33"/>
+      <c r="M10" s="31"/>
+      <c r="N10" s="31"/>
     </row>
     <row r="11" spans="1:14" ht="15" customHeight="1">
       <c r="A11" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="29">
+      <c r="B11" s="36">
         <f>SUM(B5:B10)</f>
         <v>1863</v>
       </c>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
+      <c r="C11" s="31"/>
+      <c r="D11" s="31"/>
       <c r="F11" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="G11" s="29">
+      <c r="G11" s="36">
         <f>SUM(G5:G10)</f>
         <v>0</v>
       </c>
-      <c r="H11" s="25"/>
-      <c r="I11" s="25"/>
+      <c r="H11" s="31"/>
+      <c r="I11" s="31"/>
       <c r="K11" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="L11" s="29">
+      <c r="L11" s="36">
         <f>SUM(L5:L10)</f>
         <v>0</v>
       </c>
-      <c r="M11" s="25"/>
-      <c r="N11" s="25"/>
+      <c r="M11" s="31"/>
+      <c r="N11" s="31"/>
     </row>
     <row r="12" spans="1:14" ht="15" customHeight="1">
       <c r="A12" s="9"/>
@@ -2460,44 +3103,44 @@
       <c r="N13" s="9"/>
     </row>
     <row r="25" spans="1:14" ht="15" customHeight="1">
-      <c r="A25" s="30" t="s">
+      <c r="A25" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="B25" s="25"/>
-      <c r="C25" s="25"/>
-      <c r="D25" s="25"/>
-      <c r="F25" s="30" t="s">
+      <c r="B25" s="31"/>
+      <c r="C25" s="31"/>
+      <c r="D25" s="31"/>
+      <c r="F25" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="G25" s="25"/>
-      <c r="H25" s="25"/>
-      <c r="I25" s="25"/>
-      <c r="K25" s="30" t="s">
+      <c r="G25" s="31"/>
+      <c r="H25" s="31"/>
+      <c r="I25" s="31"/>
+      <c r="K25" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="L25" s="25"/>
-      <c r="M25" s="25"/>
-      <c r="N25" s="25"/>
+      <c r="L25" s="31"/>
+      <c r="M25" s="31"/>
+      <c r="N25" s="31"/>
     </row>
     <row r="26" spans="1:14" ht="15" customHeight="1">
-      <c r="A26" s="30" t="s">
+      <c r="A26" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="B26" s="25"/>
-      <c r="C26" s="25"/>
-      <c r="D26" s="25"/>
-      <c r="F26" s="30" t="s">
+      <c r="B26" s="31"/>
+      <c r="C26" s="31"/>
+      <c r="D26" s="31"/>
+      <c r="F26" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="G26" s="25"/>
-      <c r="H26" s="25"/>
-      <c r="I26" s="25"/>
-      <c r="K26" s="30" t="s">
+      <c r="G26" s="31"/>
+      <c r="H26" s="31"/>
+      <c r="I26" s="31"/>
+      <c r="K26" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="L26" s="25"/>
-      <c r="M26" s="25"/>
-      <c r="N26" s="25"/>
+      <c r="L26" s="31"/>
+      <c r="M26" s="31"/>
+      <c r="N26" s="31"/>
     </row>
     <row r="27" spans="1:14" ht="15" customHeight="1">
       <c r="A27" s="9"/>
@@ -2514,203 +3157,203 @@
       <c r="N27" s="9"/>
     </row>
     <row r="28" spans="1:14" ht="15" customHeight="1">
-      <c r="A28" s="28" t="s">
+      <c r="A28" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="28" t="s">
+      <c r="B28" s="31"/>
+      <c r="C28" s="35" t="s">
         <v>38</v>
       </c>
-      <c r="D28" s="25"/>
-      <c r="F28" s="28" t="s">
+      <c r="D28" s="31"/>
+      <c r="F28" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="G28" s="25"/>
-      <c r="H28" s="28" t="s">
+      <c r="G28" s="31"/>
+      <c r="H28" s="35" t="s">
         <v>39</v>
       </c>
-      <c r="I28" s="25"/>
-      <c r="K28" s="28" t="s">
+      <c r="I28" s="31"/>
+      <c r="K28" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="L28" s="25"/>
-      <c r="M28" s="28" t="s">
+      <c r="L28" s="31"/>
+      <c r="M28" s="35" t="s">
         <v>40</v>
       </c>
-      <c r="N28" s="25"/>
+      <c r="N28" s="31"/>
     </row>
     <row r="29" spans="1:14" ht="15" customHeight="1">
       <c r="A29" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B29" s="27">
-        <v>0</v>
-      </c>
-      <c r="C29" s="25"/>
-      <c r="D29" s="25"/>
+      <c r="B29" s="34">
+        <v>0</v>
+      </c>
+      <c r="C29" s="31"/>
+      <c r="D29" s="31"/>
       <c r="F29" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G29" s="27"/>
-      <c r="H29" s="25"/>
-      <c r="I29" s="25"/>
+      <c r="G29" s="34"/>
+      <c r="H29" s="31"/>
+      <c r="I29" s="31"/>
       <c r="K29" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="L29" s="27">
+      <c r="L29" s="34">
         <v>14</v>
       </c>
-      <c r="M29" s="25"/>
-      <c r="N29" s="25"/>
+      <c r="M29" s="31"/>
+      <c r="N29" s="31"/>
     </row>
     <row r="30" spans="1:14" ht="15" customHeight="1">
       <c r="A30" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="B30" s="26">
-        <v>0</v>
-      </c>
-      <c r="C30" s="25"/>
-      <c r="D30" s="25"/>
+      <c r="B30" s="33">
+        <v>0</v>
+      </c>
+      <c r="C30" s="31"/>
+      <c r="D30" s="31"/>
       <c r="F30" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="G30" s="26"/>
-      <c r="H30" s="25"/>
-      <c r="I30" s="25"/>
+      <c r="G30" s="33"/>
+      <c r="H30" s="31"/>
+      <c r="I30" s="31"/>
       <c r="K30" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="L30" s="26">
+      <c r="L30" s="33">
         <v>605</v>
       </c>
-      <c r="M30" s="25"/>
-      <c r="N30" s="25"/>
+      <c r="M30" s="31"/>
+      <c r="N30" s="31"/>
     </row>
     <row r="31" spans="1:14" ht="15" customHeight="1">
       <c r="A31" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B31" s="27">
-        <v>0</v>
-      </c>
-      <c r="C31" s="25"/>
-      <c r="D31" s="25"/>
+      <c r="B31" s="34">
+        <v>0</v>
+      </c>
+      <c r="C31" s="31"/>
+      <c r="D31" s="31"/>
       <c r="F31" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G31" s="27"/>
-      <c r="H31" s="25"/>
-      <c r="I31" s="25"/>
+      <c r="G31" s="34"/>
+      <c r="H31" s="31"/>
+      <c r="I31" s="31"/>
       <c r="K31" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="L31" s="27">
+      <c r="L31" s="34">
         <v>1708</v>
       </c>
-      <c r="M31" s="25"/>
-      <c r="N31" s="25"/>
+      <c r="M31" s="31"/>
+      <c r="N31" s="31"/>
     </row>
     <row r="32" spans="1:14" ht="15" customHeight="1">
       <c r="A32" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B32" s="26">
-        <v>0</v>
-      </c>
-      <c r="C32" s="25"/>
-      <c r="D32" s="25"/>
+      <c r="B32" s="33">
+        <v>0</v>
+      </c>
+      <c r="C32" s="31"/>
+      <c r="D32" s="31"/>
       <c r="F32" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="G32" s="26"/>
-      <c r="H32" s="25"/>
-      <c r="I32" s="25"/>
+      <c r="G32" s="33"/>
+      <c r="H32" s="31"/>
+      <c r="I32" s="31"/>
       <c r="K32" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="L32" s="26">
+      <c r="L32" s="33">
         <v>1395</v>
       </c>
-      <c r="M32" s="25"/>
-      <c r="N32" s="25"/>
+      <c r="M32" s="31"/>
+      <c r="N32" s="31"/>
     </row>
     <row r="33" spans="1:14" ht="15" customHeight="1">
       <c r="A33" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B33" s="27">
-        <v>0</v>
-      </c>
-      <c r="C33" s="25"/>
-      <c r="D33" s="25"/>
+      <c r="B33" s="34">
+        <v>0</v>
+      </c>
+      <c r="C33" s="31"/>
+      <c r="D33" s="31"/>
       <c r="F33" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G33" s="27"/>
-      <c r="H33" s="25"/>
-      <c r="I33" s="25"/>
+      <c r="G33" s="34"/>
+      <c r="H33" s="31"/>
+      <c r="I33" s="31"/>
       <c r="K33" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="L33" s="27">
-        <v>0</v>
-      </c>
-      <c r="M33" s="25"/>
-      <c r="N33" s="25"/>
+      <c r="L33" s="34">
+        <v>0</v>
+      </c>
+      <c r="M33" s="31"/>
+      <c r="N33" s="31"/>
     </row>
     <row r="34" spans="1:14" ht="15" customHeight="1">
       <c r="A34" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="B34" s="26">
-        <v>0</v>
-      </c>
-      <c r="C34" s="25"/>
-      <c r="D34" s="25"/>
+      <c r="B34" s="33">
+        <v>0</v>
+      </c>
+      <c r="C34" s="31"/>
+      <c r="D34" s="31"/>
       <c r="F34" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="G34" s="26"/>
-      <c r="H34" s="25"/>
-      <c r="I34" s="25"/>
+      <c r="G34" s="33"/>
+      <c r="H34" s="31"/>
+      <c r="I34" s="31"/>
       <c r="K34" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="L34" s="26">
-        <v>0</v>
-      </c>
-      <c r="M34" s="25"/>
-      <c r="N34" s="25"/>
+      <c r="L34" s="33">
+        <v>0</v>
+      </c>
+      <c r="M34" s="31"/>
+      <c r="N34" s="31"/>
     </row>
     <row r="35" spans="1:14" ht="15" customHeight="1">
       <c r="A35" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B35" s="29">
+      <c r="B35" s="36">
         <f>SUM(B29:B34)</f>
         <v>0</v>
       </c>
-      <c r="C35" s="25"/>
-      <c r="D35" s="25"/>
+      <c r="C35" s="31"/>
+      <c r="D35" s="31"/>
       <c r="F35" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="G35" s="29">
+      <c r="G35" s="36">
         <f>SUM(G29:G34)</f>
         <v>0</v>
       </c>
-      <c r="H35" s="25"/>
-      <c r="I35" s="25"/>
+      <c r="H35" s="31"/>
+      <c r="I35" s="31"/>
       <c r="K35" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="L35" s="29">
+      <c r="L35" s="36">
         <f>SUM(L29:L34)</f>
         <v>3722</v>
       </c>
-      <c r="M35" s="25"/>
-      <c r="N35" s="25"/>
+      <c r="M35" s="31"/>
+      <c r="N35" s="31"/>
     </row>
     <row r="36" spans="1:14" ht="15" customHeight="1">
       <c r="A36" s="9"/>
@@ -2742,13 +3385,49 @@
     </row>
   </sheetData>
   <mergeCells count="66">
-    <mergeCell ref="F26:I26"/>
-    <mergeCell ref="L32:N32"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="L29:N29"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="L5:N5"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="G35:I35"/>
+    <mergeCell ref="L31:N31"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="L34:N34"/>
+    <mergeCell ref="G29:I29"/>
+    <mergeCell ref="L33:N33"/>
+    <mergeCell ref="L35:N35"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="G30:I30"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="G33:I33"/>
+    <mergeCell ref="L30:N30"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="G34:I34"/>
+    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="L10:N10"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="K25:N25"/>
+    <mergeCell ref="L9:N9"/>
+    <mergeCell ref="F25:I25"/>
+    <mergeCell ref="L6:N6"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="L8:N8"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="G11:I11"/>
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="L11:N11"/>
@@ -2765,49 +3444,13 @@
     <mergeCell ref="K2:N2"/>
     <mergeCell ref="K4:L4"/>
     <mergeCell ref="G7:I7"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="L10:N10"/>
-    <mergeCell ref="G5:I5"/>
-    <mergeCell ref="K25:N25"/>
-    <mergeCell ref="L9:N9"/>
-    <mergeCell ref="F25:I25"/>
-    <mergeCell ref="L6:N6"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="L8:N8"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="G35:I35"/>
-    <mergeCell ref="L31:N31"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="L34:N34"/>
-    <mergeCell ref="G29:I29"/>
-    <mergeCell ref="L33:N33"/>
-    <mergeCell ref="L35:N35"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="G30:I30"/>
-    <mergeCell ref="B34:D34"/>
-    <mergeCell ref="G33:I33"/>
-    <mergeCell ref="L30:N30"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="G34:I34"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="B33:D33"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="L29:N29"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="L5:N5"/>
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="L32:N32"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="C28:D28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2823,20 +3466,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15" customHeight="1">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
     </row>
     <row r="2" spans="1:4" ht="15" customHeight="1">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
     </row>
     <row r="3" spans="1:4" ht="15" customHeight="1">
       <c r="A3" s="9"/>
@@ -2845,57 +3488,57 @@
       <c r="D3" s="9"/>
     </row>
     <row r="4" spans="1:4" ht="15" customHeight="1">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="25"/>
-      <c r="C4" s="28" t="s">
+      <c r="B4" s="31"/>
+      <c r="C4" s="35" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="25"/>
+      <c r="D4" s="31"/>
     </row>
     <row r="5" spans="1:4" ht="15" customHeight="1">
       <c r="A5" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B5" s="27"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
+      <c r="B5" s="34"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="31"/>
     </row>
     <row r="6" spans="1:4" ht="15" customHeight="1">
       <c r="A6" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="B6" s="26"/>
-      <c r="C6" s="25"/>
-      <c r="D6" s="25"/>
+      <c r="B6" s="33"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="31"/>
     </row>
     <row r="7" spans="1:4" ht="15" customHeight="1">
       <c r="A7" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B7" s="27"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
+      <c r="B7" s="34"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="31"/>
     </row>
     <row r="8" spans="1:4" ht="15" customHeight="1">
       <c r="A8" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="B8" s="26"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="25"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="31"/>
+      <c r="D8" s="31"/>
     </row>
     <row r="9" spans="1:4" ht="15" customHeight="1">
       <c r="A9" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B9" s="29">
+      <c r="B9" s="36">
         <f>SUM(B5:B8)</f>
         <v>0</v>
       </c>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
+      <c r="C9" s="31"/>
+      <c r="D9" s="31"/>
     </row>
     <row r="10" spans="1:4" ht="15" customHeight="1">
       <c r="A10" s="9"/>
@@ -2939,44 +3582,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15" customHeight="1">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="F1" s="30" t="s">
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="F1" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="K1" s="30" t="s">
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="K1" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="L1" s="25"/>
-      <c r="M1" s="25"/>
-      <c r="N1" s="25"/>
+      <c r="L1" s="31"/>
+      <c r="M1" s="31"/>
+      <c r="N1" s="31"/>
     </row>
     <row r="2" spans="1:14" ht="15" customHeight="1">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="F2" s="30" t="s">
+      <c r="B2" s="31"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="F2" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
-      <c r="I2" s="25"/>
-      <c r="K2" s="30" t="s">
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
+      <c r="K2" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="L2" s="25"/>
-      <c r="M2" s="25"/>
-      <c r="N2" s="25"/>
+      <c r="L2" s="31"/>
+      <c r="M2" s="31"/>
+      <c r="N2" s="31"/>
     </row>
     <row r="3" spans="1:14" ht="15" customHeight="1">
       <c r="A3" s="9"/>
@@ -2993,219 +3636,219 @@
       <c r="N3" s="9"/>
     </row>
     <row r="4" spans="1:14" ht="15" customHeight="1">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="25"/>
-      <c r="C4" s="28" t="s">
+      <c r="B4" s="31"/>
+      <c r="C4" s="35" t="s">
         <v>53</v>
       </c>
-      <c r="D4" s="25"/>
-      <c r="F4" s="28" t="s">
+      <c r="D4" s="31"/>
+      <c r="F4" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="G4" s="25"/>
-      <c r="H4" s="28" t="s">
+      <c r="G4" s="31"/>
+      <c r="H4" s="35" t="s">
         <v>54</v>
       </c>
-      <c r="I4" s="25"/>
-      <c r="K4" s="28" t="s">
+      <c r="I4" s="31"/>
+      <c r="K4" s="35" t="s">
         <v>37</v>
       </c>
-      <c r="L4" s="25"/>
-      <c r="M4" s="28" t="s">
+      <c r="L4" s="31"/>
+      <c r="M4" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="N4" s="25"/>
+      <c r="N4" s="31"/>
     </row>
     <row r="5" spans="1:14" ht="15" customHeight="1">
       <c r="A5" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="27"/>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
+      <c r="B5" s="34"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="31"/>
       <c r="F5" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="G5" s="27"/>
-      <c r="H5" s="25"/>
-      <c r="I5" s="25"/>
+      <c r="G5" s="34"/>
+      <c r="H5" s="31"/>
+      <c r="I5" s="31"/>
       <c r="K5" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="L5" s="27"/>
-      <c r="M5" s="25"/>
-      <c r="N5" s="25"/>
+      <c r="L5" s="34"/>
+      <c r="M5" s="31"/>
+      <c r="N5" s="31"/>
     </row>
     <row r="6" spans="1:14" ht="15" customHeight="1">
       <c r="A6" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="26"/>
-      <c r="C6" s="25"/>
-      <c r="D6" s="25"/>
+      <c r="B6" s="33"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="31"/>
       <c r="F6" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="G6" s="26"/>
-      <c r="H6" s="25"/>
-      <c r="I6" s="25"/>
+      <c r="G6" s="33"/>
+      <c r="H6" s="31"/>
+      <c r="I6" s="31"/>
       <c r="K6" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="L6" s="26"/>
-      <c r="M6" s="25"/>
-      <c r="N6" s="25"/>
+      <c r="L6" s="33"/>
+      <c r="M6" s="31"/>
+      <c r="N6" s="31"/>
     </row>
     <row r="7" spans="1:14" ht="15" customHeight="1">
       <c r="A7" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B7" s="27"/>
-      <c r="C7" s="25"/>
-      <c r="D7" s="25"/>
+      <c r="B7" s="34"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="31"/>
       <c r="F7" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="G7" s="27"/>
-      <c r="H7" s="25"/>
-      <c r="I7" s="25"/>
+      <c r="G7" s="34"/>
+      <c r="H7" s="31"/>
+      <c r="I7" s="31"/>
       <c r="K7" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="L7" s="27"/>
-      <c r="M7" s="25"/>
-      <c r="N7" s="25"/>
+      <c r="L7" s="34"/>
+      <c r="M7" s="31"/>
+      <c r="N7" s="31"/>
     </row>
     <row r="8" spans="1:14" ht="15" customHeight="1">
       <c r="A8" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B8" s="26"/>
-      <c r="C8" s="25"/>
-      <c r="D8" s="25"/>
+      <c r="B8" s="33"/>
+      <c r="C8" s="31"/>
+      <c r="D8" s="31"/>
       <c r="F8" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G8" s="26"/>
-      <c r="H8" s="25"/>
-      <c r="I8" s="25"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="31"/>
+      <c r="I8" s="31"/>
       <c r="K8" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="L8" s="26"/>
-      <c r="M8" s="25"/>
-      <c r="N8" s="25"/>
+      <c r="L8" s="33"/>
+      <c r="M8" s="31"/>
+      <c r="N8" s="31"/>
     </row>
     <row r="9" spans="1:14" ht="15" customHeight="1">
       <c r="A9" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B9" s="27"/>
-      <c r="C9" s="25"/>
-      <c r="D9" s="25"/>
+      <c r="B9" s="34"/>
+      <c r="C9" s="31"/>
+      <c r="D9" s="31"/>
       <c r="F9" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="G9" s="27"/>
-      <c r="H9" s="25"/>
-      <c r="I9" s="25"/>
+      <c r="G9" s="34"/>
+      <c r="H9" s="31"/>
+      <c r="I9" s="31"/>
       <c r="K9" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="L9" s="27"/>
-      <c r="M9" s="25"/>
-      <c r="N9" s="25"/>
+      <c r="L9" s="34"/>
+      <c r="M9" s="31"/>
+      <c r="N9" s="31"/>
     </row>
     <row r="10" spans="1:14" ht="15" customHeight="1">
       <c r="A10" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="B10" s="26"/>
-      <c r="C10" s="25"/>
-      <c r="D10" s="25"/>
+      <c r="B10" s="33"/>
+      <c r="C10" s="31"/>
+      <c r="D10" s="31"/>
       <c r="F10" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="G10" s="26"/>
-      <c r="H10" s="25"/>
-      <c r="I10" s="25"/>
+      <c r="G10" s="33"/>
+      <c r="H10" s="31"/>
+      <c r="I10" s="31"/>
       <c r="K10" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L10" s="26"/>
-      <c r="M10" s="25"/>
-      <c r="N10" s="25"/>
+      <c r="L10" s="33"/>
+      <c r="M10" s="31"/>
+      <c r="N10" s="31"/>
     </row>
     <row r="11" spans="1:14" ht="15" customHeight="1">
       <c r="A11" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="27"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
+      <c r="B11" s="34"/>
+      <c r="C11" s="31"/>
+      <c r="D11" s="31"/>
       <c r="F11" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="G11" s="27"/>
-      <c r="H11" s="25"/>
-      <c r="I11" s="25"/>
+      <c r="G11" s="34"/>
+      <c r="H11" s="31"/>
+      <c r="I11" s="31"/>
       <c r="K11" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="L11" s="27"/>
-      <c r="M11" s="25"/>
-      <c r="N11" s="25"/>
+      <c r="L11" s="34"/>
+      <c r="M11" s="31"/>
+      <c r="N11" s="31"/>
     </row>
     <row r="12" spans="1:14" ht="15" customHeight="1">
       <c r="A12" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B12" s="26"/>
-      <c r="C12" s="25"/>
-      <c r="D12" s="25"/>
+      <c r="B12" s="33"/>
+      <c r="C12" s="31"/>
+      <c r="D12" s="31"/>
       <c r="F12" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="G12" s="26"/>
-      <c r="H12" s="25"/>
-      <c r="I12" s="25"/>
+      <c r="G12" s="33"/>
+      <c r="H12" s="31"/>
+      <c r="I12" s="31"/>
       <c r="K12" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="L12" s="26"/>
-      <c r="M12" s="25"/>
-      <c r="N12" s="25"/>
+      <c r="L12" s="33"/>
+      <c r="M12" s="31"/>
+      <c r="N12" s="31"/>
     </row>
     <row r="13" spans="1:14" ht="15" customHeight="1">
       <c r="A13" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="29">
+      <c r="B13" s="36">
         <f>SUM(B5:B12)</f>
         <v>0</v>
       </c>
-      <c r="C13" s="25"/>
-      <c r="D13" s="25"/>
+      <c r="C13" s="31"/>
+      <c r="D13" s="31"/>
       <c r="F13" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="G13" s="29">
+      <c r="G13" s="36">
         <f>SUM(G5:G12)</f>
         <v>0</v>
       </c>
-      <c r="H13" s="25"/>
-      <c r="I13" s="25"/>
+      <c r="H13" s="31"/>
+      <c r="I13" s="31"/>
       <c r="K13" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="L13" s="29">
+      <c r="L13" s="36">
         <f>SUM(L5:L12)</f>
         <v>0</v>
       </c>
-      <c r="M13" s="25"/>
-      <c r="N13" s="25"/>
+      <c r="M13" s="31"/>
+      <c r="N13" s="31"/>
     </row>
     <row r="14" spans="1:14" ht="15" customHeight="1">
       <c r="A14" s="9"/>
@@ -3236,44 +3879,44 @@
       <c r="N15" s="9"/>
     </row>
     <row r="25" spans="1:14" ht="15" customHeight="1">
-      <c r="A25" s="30" t="s">
+      <c r="A25" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="B25" s="25"/>
-      <c r="C25" s="25"/>
-      <c r="D25" s="25"/>
-      <c r="F25" s="30" t="s">
+      <c r="B25" s="31"/>
+      <c r="C25" s="31"/>
+      <c r="D25" s="31"/>
+      <c r="F25" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="G25" s="25"/>
-      <c r="H25" s="25"/>
-      <c r="I25" s="25"/>
-      <c r="K25" s="30" t="s">
+      <c r="G25" s="31"/>
+      <c r="H25" s="31"/>
+      <c r="I25" s="31"/>
+      <c r="K25" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="L25" s="25"/>
-      <c r="M25" s="25"/>
-      <c r="N25" s="25"/>
+      <c r="L25" s="31"/>
+      <c r="M25" s="31"/>
+      <c r="N25" s="31"/>
     </row>
     <row r="26" spans="1:14" ht="15" customHeight="1">
-      <c r="A26" s="30" t="s">
+      <c r="A26" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="B26" s="25"/>
-      <c r="C26" s="25"/>
-      <c r="D26" s="25"/>
-      <c r="F26" s="30" t="s">
+      <c r="B26" s="31"/>
+      <c r="C26" s="31"/>
+      <c r="D26" s="31"/>
+      <c r="F26" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="G26" s="25"/>
-      <c r="H26" s="25"/>
-      <c r="I26" s="25"/>
-      <c r="K26" s="30" t="s">
+      <c r="G26" s="31"/>
+      <c r="H26" s="31"/>
+      <c r="I26" s="31"/>
+      <c r="K26" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="L26" s="25"/>
-      <c r="M26" s="25"/>
-      <c r="N26" s="25"/>
+      <c r="L26" s="31"/>
+      <c r="M26" s="31"/>
+      <c r="N26" s="31"/>
     </row>
     <row r="27" spans="1:14" ht="15" customHeight="1">
       <c r="A27" s="9"/>
@@ -3290,219 +3933,219 @@
       <c r="N27" s="9"/>
     </row>
     <row r="28" spans="1:14" ht="15" customHeight="1">
-      <c r="A28" s="28" t="s">
+      <c r="A28" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="B28" s="25"/>
-      <c r="C28" s="28" t="s">
+      <c r="B28" s="31"/>
+      <c r="C28" s="35" t="s">
         <v>53</v>
       </c>
-      <c r="D28" s="25"/>
-      <c r="F28" s="28" t="s">
+      <c r="D28" s="31"/>
+      <c r="F28" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="G28" s="25"/>
-      <c r="H28" s="28" t="s">
+      <c r="G28" s="31"/>
+      <c r="H28" s="35" t="s">
         <v>54</v>
       </c>
-      <c r="I28" s="25"/>
-      <c r="K28" s="28" t="s">
+      <c r="I28" s="31"/>
+      <c r="K28" s="35" t="s">
         <v>47</v>
       </c>
-      <c r="L28" s="25"/>
-      <c r="M28" s="28" t="s">
+      <c r="L28" s="31"/>
+      <c r="M28" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="N28" s="25"/>
+      <c r="N28" s="31"/>
     </row>
     <row r="29" spans="1:14" ht="15" customHeight="1">
       <c r="A29" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B29" s="27"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="25"/>
+      <c r="B29" s="34"/>
+      <c r="C29" s="31"/>
+      <c r="D29" s="31"/>
       <c r="F29" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="G29" s="27"/>
-      <c r="H29" s="25"/>
-      <c r="I29" s="25"/>
+      <c r="G29" s="34"/>
+      <c r="H29" s="31"/>
+      <c r="I29" s="31"/>
       <c r="K29" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="L29" s="27"/>
-      <c r="M29" s="25"/>
-      <c r="N29" s="25"/>
+      <c r="L29" s="34"/>
+      <c r="M29" s="31"/>
+      <c r="N29" s="31"/>
     </row>
     <row r="30" spans="1:14" ht="15" customHeight="1">
       <c r="A30" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B30" s="26"/>
-      <c r="C30" s="25"/>
-      <c r="D30" s="25"/>
+      <c r="B30" s="33"/>
+      <c r="C30" s="31"/>
+      <c r="D30" s="31"/>
       <c r="F30" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="G30" s="26"/>
-      <c r="H30" s="25"/>
-      <c r="I30" s="25"/>
+      <c r="G30" s="33"/>
+      <c r="H30" s="31"/>
+      <c r="I30" s="31"/>
       <c r="K30" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="L30" s="26"/>
-      <c r="M30" s="25"/>
-      <c r="N30" s="25"/>
+      <c r="L30" s="33"/>
+      <c r="M30" s="31"/>
+      <c r="N30" s="31"/>
     </row>
     <row r="31" spans="1:14" ht="15" customHeight="1">
       <c r="A31" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B31" s="27"/>
-      <c r="C31" s="25"/>
-      <c r="D31" s="25"/>
+      <c r="B31" s="34"/>
+      <c r="C31" s="31"/>
+      <c r="D31" s="31"/>
       <c r="F31" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="G31" s="27"/>
-      <c r="H31" s="25"/>
-      <c r="I31" s="25"/>
+      <c r="G31" s="34"/>
+      <c r="H31" s="31"/>
+      <c r="I31" s="31"/>
       <c r="K31" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="L31" s="27"/>
-      <c r="M31" s="25"/>
-      <c r="N31" s="25"/>
+      <c r="L31" s="34"/>
+      <c r="M31" s="31"/>
+      <c r="N31" s="31"/>
     </row>
     <row r="32" spans="1:14" ht="15" customHeight="1">
       <c r="A32" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B32" s="26"/>
-      <c r="C32" s="25"/>
-      <c r="D32" s="25"/>
+      <c r="B32" s="33"/>
+      <c r="C32" s="31"/>
+      <c r="D32" s="31"/>
       <c r="F32" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G32" s="26"/>
-      <c r="H32" s="25"/>
-      <c r="I32" s="25"/>
+      <c r="G32" s="33"/>
+      <c r="H32" s="31"/>
+      <c r="I32" s="31"/>
       <c r="K32" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="L32" s="26"/>
-      <c r="M32" s="25"/>
-      <c r="N32" s="25"/>
+      <c r="L32" s="33"/>
+      <c r="M32" s="31"/>
+      <c r="N32" s="31"/>
     </row>
     <row r="33" spans="1:14" ht="15" customHeight="1">
       <c r="A33" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B33" s="27"/>
-      <c r="C33" s="25"/>
-      <c r="D33" s="25"/>
+      <c r="B33" s="34"/>
+      <c r="C33" s="31"/>
+      <c r="D33" s="31"/>
       <c r="F33" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="G33" s="27"/>
-      <c r="H33" s="25"/>
-      <c r="I33" s="25"/>
+      <c r="G33" s="34"/>
+      <c r="H33" s="31"/>
+      <c r="I33" s="31"/>
       <c r="K33" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="L33" s="27"/>
-      <c r="M33" s="25"/>
-      <c r="N33" s="25"/>
+      <c r="L33" s="34"/>
+      <c r="M33" s="31"/>
+      <c r="N33" s="31"/>
     </row>
     <row r="34" spans="1:14" ht="15" customHeight="1">
       <c r="A34" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="B34" s="26"/>
-      <c r="C34" s="25"/>
-      <c r="D34" s="25"/>
+      <c r="B34" s="33"/>
+      <c r="C34" s="31"/>
+      <c r="D34" s="31"/>
       <c r="F34" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="G34" s="26"/>
-      <c r="H34" s="25"/>
-      <c r="I34" s="25"/>
+      <c r="G34" s="33"/>
+      <c r="H34" s="31"/>
+      <c r="I34" s="31"/>
       <c r="K34" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L34" s="26"/>
-      <c r="M34" s="25"/>
-      <c r="N34" s="25"/>
+      <c r="L34" s="33"/>
+      <c r="M34" s="31"/>
+      <c r="N34" s="31"/>
     </row>
     <row r="35" spans="1:14" ht="15" customHeight="1">
       <c r="A35" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B35" s="27"/>
-      <c r="C35" s="25"/>
-      <c r="D35" s="25"/>
+      <c r="B35" s="34"/>
+      <c r="C35" s="31"/>
+      <c r="D35" s="31"/>
       <c r="F35" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="G35" s="27"/>
-      <c r="H35" s="25"/>
-      <c r="I35" s="25"/>
+      <c r="G35" s="34"/>
+      <c r="H35" s="31"/>
+      <c r="I35" s="31"/>
       <c r="K35" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="L35" s="27"/>
-      <c r="M35" s="25"/>
-      <c r="N35" s="25"/>
+      <c r="L35" s="34"/>
+      <c r="M35" s="31"/>
+      <c r="N35" s="31"/>
     </row>
     <row r="36" spans="1:14" ht="15" customHeight="1">
       <c r="A36" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B36" s="26"/>
-      <c r="C36" s="25"/>
-      <c r="D36" s="25"/>
+      <c r="B36" s="33"/>
+      <c r="C36" s="31"/>
+      <c r="D36" s="31"/>
       <c r="F36" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="G36" s="26"/>
-      <c r="H36" s="25"/>
-      <c r="I36" s="25"/>
+      <c r="G36" s="33"/>
+      <c r="H36" s="31"/>
+      <c r="I36" s="31"/>
       <c r="K36" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="L36" s="26"/>
-      <c r="M36" s="25"/>
-      <c r="N36" s="25"/>
+      <c r="L36" s="33"/>
+      <c r="M36" s="31"/>
+      <c r="N36" s="31"/>
     </row>
     <row r="37" spans="1:14" ht="15" customHeight="1">
       <c r="A37" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B37" s="29">
+      <c r="B37" s="36">
         <f>SUM(B29:B36)</f>
         <v>0</v>
       </c>
-      <c r="C37" s="25"/>
-      <c r="D37" s="25"/>
+      <c r="C37" s="31"/>
+      <c r="D37" s="31"/>
       <c r="F37" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="G37" s="29">
+      <c r="G37" s="36">
         <f>SUM(G29:G36)</f>
         <v>0</v>
       </c>
-      <c r="H37" s="25"/>
-      <c r="I37" s="25"/>
+      <c r="H37" s="31"/>
+      <c r="I37" s="31"/>
       <c r="K37" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="L37" s="29">
+      <c r="L37" s="36">
         <f>SUM(L29:L36)</f>
         <v>0</v>
       </c>
-      <c r="M37" s="25"/>
-      <c r="N37" s="25"/>
+      <c r="M37" s="31"/>
+      <c r="N37" s="31"/>
     </row>
     <row r="38" spans="1:14" ht="15" customHeight="1">
       <c r="A38" s="9"/>
@@ -3534,6 +4177,68 @@
     </row>
   </sheetData>
   <mergeCells count="78">
+    <mergeCell ref="G36:I36"/>
+    <mergeCell ref="L32:N32"/>
+    <mergeCell ref="L13:N13"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="F25:I25"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="G32:I32"/>
+    <mergeCell ref="L36:N36"/>
+    <mergeCell ref="L33:N33"/>
+    <mergeCell ref="L35:N35"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="L11:N11"/>
+    <mergeCell ref="K26:N26"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="L30:N30"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="G33:I33"/>
+    <mergeCell ref="L29:N29"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="L37:N37"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="L12:N12"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="G34:I34"/>
+    <mergeCell ref="K25:N25"/>
+    <mergeCell ref="G29:I29"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="G37:I37"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="L8:N8"/>
+    <mergeCell ref="G30:I30"/>
+    <mergeCell ref="G35:I35"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="L31:N31"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="F2:I2"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="K2:N2"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="L5:N5"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="F4:G4"/>
     <mergeCell ref="L34:N34"/>
     <mergeCell ref="L6:N6"/>
     <mergeCell ref="B33:D33"/>
@@ -3550,68 +4255,6 @@
     <mergeCell ref="B12:D12"/>
     <mergeCell ref="A26:D26"/>
     <mergeCell ref="L9:N9"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="L31:N31"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="F2:I2"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="K2:N2"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="L5:N5"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="K1:N1"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="L37:N37"/>
-    <mergeCell ref="G8:I8"/>
-    <mergeCell ref="L12:N12"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="G34:I34"/>
-    <mergeCell ref="K25:N25"/>
-    <mergeCell ref="G29:I29"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="G31:I31"/>
-    <mergeCell ref="G37:I37"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="L8:N8"/>
-    <mergeCell ref="G30:I30"/>
-    <mergeCell ref="G35:I35"/>
-    <mergeCell ref="B37:D37"/>
-    <mergeCell ref="L30:N30"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="G33:I33"/>
-    <mergeCell ref="L29:N29"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="L11:N11"/>
-    <mergeCell ref="K26:N26"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="G5:I5"/>
-    <mergeCell ref="G36:I36"/>
-    <mergeCell ref="L32:N32"/>
-    <mergeCell ref="L13:N13"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="C28:D28"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="H28:I28"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="F25:I25"/>
-    <mergeCell ref="B36:D36"/>
-    <mergeCell ref="G32:I32"/>
-    <mergeCell ref="L36:N36"/>
-    <mergeCell ref="L33:N33"/>
-    <mergeCell ref="L35:N35"/>
-    <mergeCell ref="B34:D34"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3659,7 +4302,7 @@
         <v>49</v>
       </c>
       <c r="E2" s="18">
-        <v>180</v>
+        <v>165</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -3693,7 +4336,7 @@
         <v>49</v>
       </c>
       <c r="E4" s="18">
-        <v>180</v>
+        <v>165</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -3727,7 +4370,7 @@
         <v>49</v>
       </c>
       <c r="E6" s="18">
-        <v>180</v>
+        <v>165</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -4059,7 +4702,7 @@
         <v>49</v>
       </c>
       <c r="E26" s="18">
-        <v>180</v>
+        <v>165</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -4093,7 +4736,7 @@
         <v>49</v>
       </c>
       <c r="E28" s="18">
-        <v>180</v>
+        <v>165</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -4127,7 +4770,7 @@
         <v>49</v>
       </c>
       <c r="E30" s="18">
-        <v>180</v>
+        <v>165</v>
       </c>
     </row>
     <row r="31" spans="1:5">

</xml_diff>

<commit_message>
Atualiza disponibilidade do app Granel
Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/disponibilidade.xlsx
+++ b/disponibilidade.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rafael.germano\Documents\Rafael Germano\Codex\2026-05-19\app disponiblidade\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8A68365-18B9-4B86-A3DE-0233314273AE}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{089315A4-7ED5-40B3-AD6B-5C63B769879F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instrucoes" sheetId="1" r:id="rId1"/>
@@ -453,9 +453,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -466,6 +463,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="4" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -793,7 +793,7 @@
       </c>
       <c r="B5" s="21">
         <f>SUM(B6:B7)</f>
-        <v>2300</v>
+        <v>700</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>20</v>
@@ -807,16 +807,14 @@
       </c>
       <c r="L5" s="14">
         <f>SUM(L6:L7)</f>
-        <v>2600</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="15" customHeight="1">
       <c r="A6" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="14">
-        <v>1500</v>
-      </c>
+      <c r="B6" s="14"/>
       <c r="F6" s="7" t="s">
         <v>21</v>
       </c>
@@ -824,16 +822,14 @@
       <c r="K6" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="L6" s="14">
-        <v>2600</v>
-      </c>
+      <c r="L6" s="14"/>
     </row>
     <row r="7" spans="1:14" ht="15" customHeight="1">
       <c r="A7" s="7" t="s">
         <v>22</v>
       </c>
       <c r="B7" s="14">
-        <v>800</v>
+        <v>700</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>22</v>
@@ -864,7 +860,7 @@
       </c>
       <c r="L8" s="15">
         <f>SUM(L9:L10)</f>
-        <v>350</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="15" customHeight="1">
@@ -880,7 +876,7 @@
         <v>21</v>
       </c>
       <c r="L9" s="15">
-        <v>350</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="15" customHeight="1">
@@ -968,7 +964,7 @@
       </c>
       <c r="L14" s="15">
         <f>SUM(L15:L16)</f>
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="15" customHeight="1">
@@ -983,7 +979,9 @@
       <c r="K15" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="L15" s="15"/>
+      <c r="L15" s="15">
+        <v>40</v>
+      </c>
     </row>
     <row r="16" spans="1:14" ht="15" customHeight="1">
       <c r="A16" s="9" t="s">
@@ -1158,14 +1156,14 @@
       </c>
       <c r="B26" s="15">
         <f>SUM(B27:B28)</f>
-        <v>1100</v>
+        <v>1400</v>
       </c>
       <c r="F26" s="9" t="s">
         <v>29</v>
       </c>
       <c r="G26" s="15">
         <f>SUM(G27:G28)</f>
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="K26" s="9" t="s">
         <v>29</v>
@@ -1183,7 +1181,9 @@
       <c r="F27" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="G27" s="15"/>
+      <c r="G27" s="15">
+        <v>300</v>
+      </c>
       <c r="K27" s="9" t="s">
         <v>21</v>
       </c>
@@ -1194,7 +1194,7 @@
         <v>22</v>
       </c>
       <c r="B28" s="15">
-        <v>1100</v>
+        <v>1400</v>
       </c>
       <c r="F28" s="9" t="s">
         <v>22</v>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="L29" s="14">
         <f>SUM(L30:L31)</f>
-        <v>680</v>
+        <v>500</v>
       </c>
     </row>
     <row r="30" spans="1:12" ht="15" customHeight="1">
@@ -1241,7 +1241,7 @@
         <v>21</v>
       </c>
       <c r="L30" s="14">
-        <v>680</v>
+        <v>500</v>
       </c>
     </row>
     <row r="31" spans="1:12" ht="15" customHeight="1">
@@ -1380,7 +1380,7 @@
       </c>
       <c r="L38" s="23">
         <f>SUM(L39:L40)</f>
-        <v>50</v>
+        <v>300</v>
       </c>
     </row>
     <row r="39" spans="1:14" ht="15" customHeight="1">
@@ -1398,7 +1398,7 @@
         <v>21</v>
       </c>
       <c r="L39" s="15">
-        <v>50</v>
+        <v>300</v>
       </c>
     </row>
     <row r="40" spans="1:14" ht="15" customHeight="1">
@@ -1421,21 +1421,21 @@
       </c>
       <c r="B41" s="13">
         <f>SUM(B5,B8,B11,B14,B17,B20,B23,B26,B29,B32,B35,B38)</f>
-        <v>3540</v>
+        <v>2240</v>
       </c>
       <c r="F41" s="8" t="s">
         <v>34</v>
       </c>
       <c r="G41" s="13">
         <f>SUM(G5,G8,G11,G14,G17,G20,G23,G26,G29,G32,G35,G38)</f>
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="K41" s="8" t="s">
         <v>34</v>
       </c>
       <c r="L41" s="13">
         <f>SUM(L5,L8,L11,L14,L17,L20,L23,L26,L29,L32,L35,L38)</f>
-        <v>3680</v>
+        <v>940</v>
       </c>
     </row>
     <row r="42" spans="1:14" ht="15" customHeight="1">
@@ -1698,7 +1698,7 @@
       </c>
       <c r="L62" s="15">
         <f>SUM(L63:L64)</f>
-        <v>0</v>
+        <v>190</v>
       </c>
     </row>
     <row r="63" spans="1:14" ht="15" customHeight="1">
@@ -1715,7 +1715,9 @@
       <c r="K63" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="L63" s="15"/>
+      <c r="L63" s="15">
+        <v>190</v>
+      </c>
     </row>
     <row r="64" spans="1:14" ht="15" customHeight="1">
       <c r="A64" s="9" t="s">
@@ -2161,7 +2163,7 @@
       </c>
       <c r="L89" s="13">
         <f>SUM(L53,L56,L59,L62,L65,L68,L71,L74,L77,L80,L83,L86)</f>
-        <v>0</v>
+        <v>190</v>
       </c>
     </row>
     <row r="90" spans="1:14" ht="15" customHeight="1">
@@ -2827,19 +2829,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15" customHeight="1">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="38" t="s">
         <v>15</v>
       </c>
       <c r="B1" s="33"/>
       <c r="C1" s="33"/>
       <c r="D1" s="33"/>
-      <c r="F1" s="34" t="s">
+      <c r="F1" s="38" t="s">
         <v>15</v>
       </c>
       <c r="G1" s="33"/>
       <c r="H1" s="33"/>
       <c r="I1" s="33"/>
-      <c r="K1" s="34" t="s">
+      <c r="K1" s="38" t="s">
         <v>15</v>
       </c>
       <c r="L1" s="33"/>
@@ -2847,19 +2849,19 @@
       <c r="N1" s="33"/>
     </row>
     <row r="2" spans="1:14" ht="15" customHeight="1">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="38" t="s">
         <v>36</v>
       </c>
       <c r="B2" s="33"/>
       <c r="C2" s="33"/>
       <c r="D2" s="33"/>
-      <c r="F2" s="34" t="s">
+      <c r="F2" s="38" t="s">
         <v>36</v>
       </c>
       <c r="G2" s="33"/>
       <c r="H2" s="33"/>
       <c r="I2" s="33"/>
-      <c r="K2" s="34" t="s">
+      <c r="K2" s="38" t="s">
         <v>36</v>
       </c>
       <c r="L2" s="33"/>
@@ -2881,27 +2883,27 @@
       <c r="N3" s="9"/>
     </row>
     <row r="4" spans="1:14" ht="15" customHeight="1">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="36" t="s">
         <v>37</v>
       </c>
       <c r="B4" s="33"/>
-      <c r="C4" s="37" t="s">
+      <c r="C4" s="36" t="s">
         <v>38</v>
       </c>
       <c r="D4" s="33"/>
-      <c r="F4" s="37" t="s">
+      <c r="F4" s="36" t="s">
         <v>37</v>
       </c>
       <c r="G4" s="33"/>
-      <c r="H4" s="37" t="s">
+      <c r="H4" s="36" t="s">
         <v>39</v>
       </c>
       <c r="I4" s="33"/>
-      <c r="K4" s="37" t="s">
+      <c r="K4" s="36" t="s">
         <v>37</v>
       </c>
       <c r="L4" s="33"/>
-      <c r="M4" s="37" t="s">
+      <c r="M4" s="36" t="s">
         <v>40</v>
       </c>
       <c r="N4" s="33"/>
@@ -2910,21 +2912,21 @@
       <c r="A5" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="36">
-        <v>0</v>
-      </c>
-      <c r="C5" s="36"/>
-      <c r="D5" s="36"/>
+      <c r="B5" s="35">
+        <v>0</v>
+      </c>
+      <c r="C5" s="35"/>
+      <c r="D5" s="35"/>
       <c r="F5" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G5" s="36"/>
+      <c r="G5" s="35"/>
       <c r="H5" s="33"/>
       <c r="I5" s="33"/>
       <c r="K5" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="L5" s="36"/>
+      <c r="L5" s="35"/>
       <c r="M5" s="33"/>
       <c r="N5" s="33"/>
     </row>
@@ -2932,21 +2934,21 @@
       <c r="A6" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="35">
-        <v>0</v>
-      </c>
-      <c r="C6" s="35"/>
-      <c r="D6" s="35"/>
+      <c r="B6" s="34">
+        <v>0</v>
+      </c>
+      <c r="C6" s="34"/>
+      <c r="D6" s="34"/>
       <c r="F6" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="G6" s="35"/>
+      <c r="G6" s="34"/>
       <c r="H6" s="33"/>
       <c r="I6" s="33"/>
       <c r="K6" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="L6" s="35"/>
+      <c r="L6" s="34"/>
       <c r="M6" s="33"/>
       <c r="N6" s="33"/>
     </row>
@@ -2954,21 +2956,21 @@
       <c r="A7" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B7" s="36">
-        <v>0</v>
-      </c>
-      <c r="C7" s="36"/>
-      <c r="D7" s="36"/>
+      <c r="B7" s="35">
+        <v>0</v>
+      </c>
+      <c r="C7" s="35"/>
+      <c r="D7" s="35"/>
       <c r="F7" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G7" s="36"/>
+      <c r="G7" s="35"/>
       <c r="H7" s="33"/>
       <c r="I7" s="33"/>
       <c r="K7" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="L7" s="36"/>
+      <c r="L7" s="35"/>
       <c r="M7" s="33"/>
       <c r="N7" s="33"/>
     </row>
@@ -2976,21 +2978,21 @@
       <c r="A8" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B8" s="35">
-        <v>0</v>
-      </c>
-      <c r="C8" s="35"/>
-      <c r="D8" s="35"/>
+      <c r="B8" s="34">
+        <v>0</v>
+      </c>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
       <c r="F8" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="G8" s="35"/>
+      <c r="G8" s="34"/>
       <c r="H8" s="33"/>
       <c r="I8" s="33"/>
       <c r="K8" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="L8" s="35"/>
+      <c r="L8" s="34"/>
       <c r="M8" s="33"/>
       <c r="N8" s="33"/>
     </row>
@@ -2998,21 +3000,21 @@
       <c r="A9" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B9" s="36">
-        <v>0</v>
-      </c>
-      <c r="C9" s="36"/>
-      <c r="D9" s="36"/>
+      <c r="B9" s="35">
+        <v>0</v>
+      </c>
+      <c r="C9" s="35"/>
+      <c r="D9" s="35"/>
       <c r="F9" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G9" s="36"/>
+      <c r="G9" s="35"/>
       <c r="H9" s="33"/>
       <c r="I9" s="33"/>
       <c r="K9" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="L9" s="36"/>
+      <c r="L9" s="35"/>
       <c r="M9" s="33"/>
       <c r="N9" s="33"/>
     </row>
@@ -3020,21 +3022,21 @@
       <c r="A10" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="B10" s="35">
-        <v>0</v>
-      </c>
-      <c r="C10" s="35"/>
-      <c r="D10" s="35"/>
+      <c r="B10" s="34">
+        <v>0</v>
+      </c>
+      <c r="C10" s="34"/>
+      <c r="D10" s="34"/>
       <c r="F10" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="G10" s="35"/>
+      <c r="G10" s="34"/>
       <c r="H10" s="33"/>
       <c r="I10" s="33"/>
       <c r="K10" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="L10" s="35"/>
+      <c r="L10" s="34"/>
       <c r="M10" s="33"/>
       <c r="N10" s="33"/>
     </row>
@@ -3042,7 +3044,7 @@
       <c r="A11" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="38">
+      <c r="B11" s="37">
         <f>SUM(B5:B10)</f>
         <v>0</v>
       </c>
@@ -3051,7 +3053,7 @@
       <c r="F11" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="G11" s="38">
+      <c r="G11" s="37">
         <f>SUM(G5:G10)</f>
         <v>0</v>
       </c>
@@ -3060,7 +3062,7 @@
       <c r="K11" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="L11" s="38">
+      <c r="L11" s="37">
         <f>SUM(L5:L10)</f>
         <v>0</v>
       </c>
@@ -3096,19 +3098,19 @@
       <c r="N13" s="9"/>
     </row>
     <row r="25" spans="1:14" ht="15" customHeight="1">
-      <c r="A25" s="34" t="s">
+      <c r="A25" s="38" t="s">
         <v>15</v>
       </c>
       <c r="B25" s="33"/>
       <c r="C25" s="33"/>
       <c r="D25" s="33"/>
-      <c r="F25" s="34" t="s">
+      <c r="F25" s="38" t="s">
         <v>15</v>
       </c>
       <c r="G25" s="33"/>
       <c r="H25" s="33"/>
       <c r="I25" s="33"/>
-      <c r="K25" s="34" t="s">
+      <c r="K25" s="38" t="s">
         <v>15</v>
       </c>
       <c r="L25" s="33"/>
@@ -3116,19 +3118,19 @@
       <c r="N25" s="33"/>
     </row>
     <row r="26" spans="1:14" ht="15" customHeight="1">
-      <c r="A26" s="34" t="s">
+      <c r="A26" s="38" t="s">
         <v>36</v>
       </c>
       <c r="B26" s="33"/>
       <c r="C26" s="33"/>
       <c r="D26" s="33"/>
-      <c r="F26" s="34" t="s">
+      <c r="F26" s="38" t="s">
         <v>36</v>
       </c>
       <c r="G26" s="33"/>
       <c r="H26" s="33"/>
       <c r="I26" s="33"/>
-      <c r="K26" s="34" t="s">
+      <c r="K26" s="38" t="s">
         <v>36</v>
       </c>
       <c r="L26" s="33"/>
@@ -3150,27 +3152,27 @@
       <c r="N27" s="9"/>
     </row>
     <row r="28" spans="1:14" ht="15" customHeight="1">
-      <c r="A28" s="37" t="s">
+      <c r="A28" s="36" t="s">
         <v>47</v>
       </c>
       <c r="B28" s="33"/>
-      <c r="C28" s="37" t="s">
+      <c r="C28" s="36" t="s">
         <v>38</v>
       </c>
       <c r="D28" s="33"/>
-      <c r="F28" s="37" t="s">
+      <c r="F28" s="36" t="s">
         <v>47</v>
       </c>
       <c r="G28" s="33"/>
-      <c r="H28" s="37" t="s">
+      <c r="H28" s="36" t="s">
         <v>39</v>
       </c>
       <c r="I28" s="33"/>
-      <c r="K28" s="37" t="s">
+      <c r="K28" s="36" t="s">
         <v>47</v>
       </c>
       <c r="L28" s="33"/>
-      <c r="M28" s="37" t="s">
+      <c r="M28" s="36" t="s">
         <v>40</v>
       </c>
       <c r="N28" s="33"/>
@@ -3179,7 +3181,7 @@
       <c r="A29" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="B29" s="36">
+      <c r="B29" s="35">
         <v>0</v>
       </c>
       <c r="C29" s="33"/>
@@ -3187,23 +3189,23 @@
       <c r="F29" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="G29" s="36"/>
+      <c r="G29" s="35"/>
       <c r="H29" s="33"/>
       <c r="I29" s="33"/>
       <c r="K29" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="L29" s="36">
-        <v>0</v>
-      </c>
-      <c r="M29" s="36"/>
-      <c r="N29" s="36"/>
+      <c r="L29" s="35">
+        <v>0</v>
+      </c>
+      <c r="M29" s="35"/>
+      <c r="N29" s="35"/>
     </row>
     <row r="30" spans="1:14" ht="15" customHeight="1">
       <c r="A30" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="B30" s="35">
+      <c r="B30" s="34">
         <v>0</v>
       </c>
       <c r="C30" s="33"/>
@@ -3211,23 +3213,23 @@
       <c r="F30" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="G30" s="35"/>
+      <c r="G30" s="34"/>
       <c r="H30" s="33"/>
       <c r="I30" s="33"/>
       <c r="K30" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="L30" s="35">
-        <v>0</v>
-      </c>
-      <c r="M30" s="35"/>
-      <c r="N30" s="35"/>
+      <c r="L30" s="34">
+        <v>0</v>
+      </c>
+      <c r="M30" s="34"/>
+      <c r="N30" s="34"/>
     </row>
     <row r="31" spans="1:14" ht="15" customHeight="1">
       <c r="A31" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B31" s="36">
+      <c r="B31" s="35">
         <v>0</v>
       </c>
       <c r="C31" s="33"/>
@@ -3235,23 +3237,23 @@
       <c r="F31" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G31" s="36"/>
+      <c r="G31" s="35"/>
       <c r="H31" s="33"/>
       <c r="I31" s="33"/>
       <c r="K31" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="L31" s="36">
-        <v>0</v>
-      </c>
-      <c r="M31" s="36"/>
-      <c r="N31" s="36"/>
+      <c r="L31" s="35">
+        <v>0</v>
+      </c>
+      <c r="M31" s="35"/>
+      <c r="N31" s="35"/>
     </row>
     <row r="32" spans="1:14" ht="15" customHeight="1">
       <c r="A32" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="B32" s="35">
+      <c r="B32" s="34">
         <v>0</v>
       </c>
       <c r="C32" s="33"/>
@@ -3259,23 +3261,23 @@
       <c r="F32" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="G32" s="35"/>
+      <c r="G32" s="34"/>
       <c r="H32" s="33"/>
       <c r="I32" s="33"/>
       <c r="K32" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="L32" s="35">
-        <v>0</v>
-      </c>
-      <c r="M32" s="35"/>
-      <c r="N32" s="35"/>
+      <c r="L32" s="34">
+        <v>0</v>
+      </c>
+      <c r="M32" s="34"/>
+      <c r="N32" s="34"/>
     </row>
     <row r="33" spans="1:14" ht="15" customHeight="1">
       <c r="A33" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B33" s="36">
+      <c r="B33" s="35">
         <v>0</v>
       </c>
       <c r="C33" s="33"/>
@@ -3283,23 +3285,23 @@
       <c r="F33" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="G33" s="36"/>
+      <c r="G33" s="35"/>
       <c r="H33" s="33"/>
       <c r="I33" s="33"/>
       <c r="K33" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="L33" s="36">
-        <v>0</v>
-      </c>
-      <c r="M33" s="36"/>
-      <c r="N33" s="36"/>
+      <c r="L33" s="35">
+        <v>0</v>
+      </c>
+      <c r="M33" s="35"/>
+      <c r="N33" s="35"/>
     </row>
     <row r="34" spans="1:14" ht="15" customHeight="1">
       <c r="A34" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="B34" s="35">
+      <c r="B34" s="34">
         <v>0</v>
       </c>
       <c r="C34" s="33"/>
@@ -3307,13 +3309,13 @@
       <c r="F34" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="G34" s="35"/>
+      <c r="G34" s="34"/>
       <c r="H34" s="33"/>
       <c r="I34" s="33"/>
       <c r="K34" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="L34" s="35">
+      <c r="L34" s="34">
         <v>0</v>
       </c>
       <c r="M34" s="33"/>
@@ -3323,7 +3325,7 @@
       <c r="A35" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B35" s="38">
+      <c r="B35" s="37">
         <f>SUM(B29:B34)</f>
         <v>0</v>
       </c>
@@ -3332,7 +3334,7 @@
       <c r="F35" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="G35" s="38">
+      <c r="G35" s="37">
         <f>SUM(G29:G34)</f>
         <v>0</v>
       </c>
@@ -3341,7 +3343,7 @@
       <c r="K35" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="L35" s="38">
+      <c r="L35" s="37">
         <f>SUM(L29:L34)</f>
         <v>0</v>
       </c>
@@ -3378,6 +3380,56 @@
     </row>
   </sheetData>
   <mergeCells count="66">
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="L32:N32"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="C28:D28"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="L11:N11"/>
+    <mergeCell ref="G32:I32"/>
+    <mergeCell ref="K26:N26"/>
+    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="L7:N7"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="F2:I2"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="K2:N2"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="L10:N10"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="K25:N25"/>
+    <mergeCell ref="L9:N9"/>
+    <mergeCell ref="F25:I25"/>
+    <mergeCell ref="L6:N6"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="L8:N8"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="G35:I35"/>
+    <mergeCell ref="L31:N31"/>
+    <mergeCell ref="B30:D30"/>
+    <mergeCell ref="L34:N34"/>
+    <mergeCell ref="G29:I29"/>
+    <mergeCell ref="L33:N33"/>
+    <mergeCell ref="L35:N35"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="G30:I30"/>
+    <mergeCell ref="B34:D34"/>
+    <mergeCell ref="G33:I33"/>
+    <mergeCell ref="L30:N30"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="G34:I34"/>
     <mergeCell ref="B6:D6"/>
     <mergeCell ref="B33:D33"/>
     <mergeCell ref="B10:D10"/>
@@ -3394,56 +3446,6 @@
     <mergeCell ref="A25:D25"/>
     <mergeCell ref="F28:G28"/>
     <mergeCell ref="H28:I28"/>
-    <mergeCell ref="G35:I35"/>
-    <mergeCell ref="L31:N31"/>
-    <mergeCell ref="B30:D30"/>
-    <mergeCell ref="L34:N34"/>
-    <mergeCell ref="G29:I29"/>
-    <mergeCell ref="L33:N33"/>
-    <mergeCell ref="L35:N35"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="G30:I30"/>
-    <mergeCell ref="B34:D34"/>
-    <mergeCell ref="G33:I33"/>
-    <mergeCell ref="L30:N30"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="G34:I34"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="L10:N10"/>
-    <mergeCell ref="G5:I5"/>
-    <mergeCell ref="K25:N25"/>
-    <mergeCell ref="L9:N9"/>
-    <mergeCell ref="F25:I25"/>
-    <mergeCell ref="L6:N6"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="L8:N8"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="L11:N11"/>
-    <mergeCell ref="G32:I32"/>
-    <mergeCell ref="K26:N26"/>
-    <mergeCell ref="G31:I31"/>
-    <mergeCell ref="K1:N1"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="L7:N7"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="F2:I2"/>
-    <mergeCell ref="G8:I8"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="K2:N2"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="F26:I26"/>
-    <mergeCell ref="L32:N32"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="C28:D28"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3459,7 +3461,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15" customHeight="1">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="38" t="s">
         <v>15</v>
       </c>
       <c r="B1" s="33"/>
@@ -3467,7 +3469,7 @@
       <c r="D1" s="33"/>
     </row>
     <row r="2" spans="1:4" ht="15" customHeight="1">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="38" t="s">
         <v>36</v>
       </c>
       <c r="B2" s="33"/>
@@ -3481,11 +3483,11 @@
       <c r="D3" s="9"/>
     </row>
     <row r="4" spans="1:4" ht="15" customHeight="1">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="36" t="s">
         <v>19</v>
       </c>
       <c r="B4" s="33"/>
-      <c r="C4" s="37" t="s">
+      <c r="C4" s="36" t="s">
         <v>48</v>
       </c>
       <c r="D4" s="33"/>
@@ -3494,7 +3496,7 @@
       <c r="A5" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="B5" s="36"/>
+      <c r="B5" s="35"/>
       <c r="C5" s="33"/>
       <c r="D5" s="33"/>
     </row>
@@ -3502,7 +3504,7 @@
       <c r="A6" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="B6" s="35"/>
+      <c r="B6" s="34"/>
       <c r="C6" s="33"/>
       <c r="D6" s="33"/>
     </row>
@@ -3510,7 +3512,7 @@
       <c r="A7" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="B7" s="36"/>
+      <c r="B7" s="35"/>
       <c r="C7" s="33"/>
       <c r="D7" s="33"/>
     </row>
@@ -3518,7 +3520,7 @@
       <c r="A8" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="B8" s="35"/>
+      <c r="B8" s="34"/>
       <c r="C8" s="33"/>
       <c r="D8" s="33"/>
     </row>
@@ -3526,7 +3528,7 @@
       <c r="A9" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B9" s="38">
+      <c r="B9" s="37">
         <f>SUM(B5:B8)</f>
         <v>0</v>
       </c>
@@ -3575,19 +3577,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="15" customHeight="1">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="38" t="s">
         <v>15</v>
       </c>
       <c r="B1" s="33"/>
       <c r="C1" s="33"/>
       <c r="D1" s="33"/>
-      <c r="F1" s="34" t="s">
+      <c r="F1" s="38" t="s">
         <v>15</v>
       </c>
       <c r="G1" s="33"/>
       <c r="H1" s="33"/>
       <c r="I1" s="33"/>
-      <c r="K1" s="34" t="s">
+      <c r="K1" s="38" t="s">
         <v>15</v>
       </c>
       <c r="L1" s="33"/>
@@ -3595,19 +3597,19 @@
       <c r="N1" s="33"/>
     </row>
     <row r="2" spans="1:14" ht="15" customHeight="1">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="38" t="s">
         <v>36</v>
       </c>
       <c r="B2" s="33"/>
       <c r="C2" s="33"/>
       <c r="D2" s="33"/>
-      <c r="F2" s="34" t="s">
+      <c r="F2" s="38" t="s">
         <v>36</v>
       </c>
       <c r="G2" s="33"/>
       <c r="H2" s="33"/>
       <c r="I2" s="33"/>
-      <c r="K2" s="34" t="s">
+      <c r="K2" s="38" t="s">
         <v>36</v>
       </c>
       <c r="L2" s="33"/>
@@ -3629,27 +3631,27 @@
       <c r="N3" s="9"/>
     </row>
     <row r="4" spans="1:14" ht="15" customHeight="1">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="36" t="s">
         <v>37</v>
       </c>
       <c r="B4" s="33"/>
-      <c r="C4" s="37" t="s">
+      <c r="C4" s="36" t="s">
         <v>53</v>
       </c>
       <c r="D4" s="33"/>
-      <c r="F4" s="37" t="s">
+      <c r="F4" s="36" t="s">
         <v>37</v>
       </c>
       <c r="G4" s="33"/>
-      <c r="H4" s="37" t="s">
+      <c r="H4" s="36" t="s">
         <v>54</v>
       </c>
       <c r="I4" s="33"/>
-      <c r="K4" s="37" t="s">
+      <c r="K4" s="36" t="s">
         <v>37</v>
       </c>
       <c r="L4" s="33"/>
-      <c r="M4" s="37" t="s">
+      <c r="M4" s="36" t="s">
         <v>55</v>
       </c>
       <c r="N4" s="33"/>
@@ -3658,19 +3660,19 @@
       <c r="A5" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="36"/>
+      <c r="B5" s="35"/>
       <c r="C5" s="33"/>
       <c r="D5" s="33"/>
       <c r="F5" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="G5" s="36"/>
+      <c r="G5" s="35"/>
       <c r="H5" s="33"/>
       <c r="I5" s="33"/>
       <c r="K5" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="L5" s="36"/>
+      <c r="L5" s="35"/>
       <c r="M5" s="33"/>
       <c r="N5" s="33"/>
     </row>
@@ -3678,19 +3680,19 @@
       <c r="A6" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="35"/>
+      <c r="B6" s="34"/>
       <c r="C6" s="33"/>
       <c r="D6" s="33"/>
       <c r="F6" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="G6" s="35"/>
+      <c r="G6" s="34"/>
       <c r="H6" s="33"/>
       <c r="I6" s="33"/>
       <c r="K6" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="L6" s="35"/>
+      <c r="L6" s="34"/>
       <c r="M6" s="33"/>
       <c r="N6" s="33"/>
     </row>
@@ -3698,19 +3700,19 @@
       <c r="A7" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B7" s="36"/>
+      <c r="B7" s="35"/>
       <c r="C7" s="33"/>
       <c r="D7" s="33"/>
       <c r="F7" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="G7" s="36"/>
+      <c r="G7" s="35"/>
       <c r="H7" s="33"/>
       <c r="I7" s="33"/>
       <c r="K7" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="L7" s="36"/>
+      <c r="L7" s="35"/>
       <c r="M7" s="33"/>
       <c r="N7" s="33"/>
     </row>
@@ -3718,19 +3720,19 @@
       <c r="A8" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B8" s="35"/>
+      <c r="B8" s="34"/>
       <c r="C8" s="33"/>
       <c r="D8" s="33"/>
       <c r="F8" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G8" s="35"/>
+      <c r="G8" s="34"/>
       <c r="H8" s="33"/>
       <c r="I8" s="33"/>
       <c r="K8" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="L8" s="35"/>
+      <c r="L8" s="34"/>
       <c r="M8" s="33"/>
       <c r="N8" s="33"/>
     </row>
@@ -3738,19 +3740,19 @@
       <c r="A9" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B9" s="36"/>
+      <c r="B9" s="35"/>
       <c r="C9" s="33"/>
       <c r="D9" s="33"/>
       <c r="F9" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="G9" s="36"/>
+      <c r="G9" s="35"/>
       <c r="H9" s="33"/>
       <c r="I9" s="33"/>
       <c r="K9" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="L9" s="36"/>
+      <c r="L9" s="35"/>
       <c r="M9" s="33"/>
       <c r="N9" s="33"/>
     </row>
@@ -3758,19 +3760,19 @@
       <c r="A10" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="B10" s="35"/>
+      <c r="B10" s="34"/>
       <c r="C10" s="33"/>
       <c r="D10" s="33"/>
       <c r="F10" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="G10" s="35"/>
+      <c r="G10" s="34"/>
       <c r="H10" s="33"/>
       <c r="I10" s="33"/>
       <c r="K10" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L10" s="35"/>
+      <c r="L10" s="34"/>
       <c r="M10" s="33"/>
       <c r="N10" s="33"/>
     </row>
@@ -3778,19 +3780,19 @@
       <c r="A11" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B11" s="36"/>
+      <c r="B11" s="35"/>
       <c r="C11" s="33"/>
       <c r="D11" s="33"/>
       <c r="F11" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="G11" s="36"/>
+      <c r="G11" s="35"/>
       <c r="H11" s="33"/>
       <c r="I11" s="33"/>
       <c r="K11" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="L11" s="36"/>
+      <c r="L11" s="35"/>
       <c r="M11" s="33"/>
       <c r="N11" s="33"/>
     </row>
@@ -3798,19 +3800,19 @@
       <c r="A12" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B12" s="35"/>
+      <c r="B12" s="34"/>
       <c r="C12" s="33"/>
       <c r="D12" s="33"/>
       <c r="F12" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="G12" s="35"/>
+      <c r="G12" s="34"/>
       <c r="H12" s="33"/>
       <c r="I12" s="33"/>
       <c r="K12" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="L12" s="35"/>
+      <c r="L12" s="34"/>
       <c r="M12" s="33"/>
       <c r="N12" s="33"/>
     </row>
@@ -3818,7 +3820,7 @@
       <c r="A13" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="38">
+      <c r="B13" s="37">
         <f>SUM(B5:B12)</f>
         <v>0</v>
       </c>
@@ -3827,7 +3829,7 @@
       <c r="F13" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="G13" s="38">
+      <c r="G13" s="37">
         <f>SUM(G5:G12)</f>
         <v>0</v>
       </c>
@@ -3836,7 +3838,7 @@
       <c r="K13" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="L13" s="38">
+      <c r="L13" s="37">
         <f>SUM(L5:L12)</f>
         <v>0</v>
       </c>
@@ -3872,19 +3874,19 @@
       <c r="N15" s="9"/>
     </row>
     <row r="25" spans="1:14" ht="15" customHeight="1">
-      <c r="A25" s="34" t="s">
+      <c r="A25" s="38" t="s">
         <v>15</v>
       </c>
       <c r="B25" s="33"/>
       <c r="C25" s="33"/>
       <c r="D25" s="33"/>
-      <c r="F25" s="34" t="s">
+      <c r="F25" s="38" t="s">
         <v>15</v>
       </c>
       <c r="G25" s="33"/>
       <c r="H25" s="33"/>
       <c r="I25" s="33"/>
-      <c r="K25" s="34" t="s">
+      <c r="K25" s="38" t="s">
         <v>15</v>
       </c>
       <c r="L25" s="33"/>
@@ -3892,19 +3894,19 @@
       <c r="N25" s="33"/>
     </row>
     <row r="26" spans="1:14" ht="15" customHeight="1">
-      <c r="A26" s="34" t="s">
+      <c r="A26" s="38" t="s">
         <v>36</v>
       </c>
       <c r="B26" s="33"/>
       <c r="C26" s="33"/>
       <c r="D26" s="33"/>
-      <c r="F26" s="34" t="s">
+      <c r="F26" s="38" t="s">
         <v>36</v>
       </c>
       <c r="G26" s="33"/>
       <c r="H26" s="33"/>
       <c r="I26" s="33"/>
-      <c r="K26" s="34" t="s">
+      <c r="K26" s="38" t="s">
         <v>36</v>
       </c>
       <c r="L26" s="33"/>
@@ -3926,27 +3928,27 @@
       <c r="N27" s="9"/>
     </row>
     <row r="28" spans="1:14" ht="15" customHeight="1">
-      <c r="A28" s="37" t="s">
+      <c r="A28" s="36" t="s">
         <v>47</v>
       </c>
       <c r="B28" s="33"/>
-      <c r="C28" s="37" t="s">
+      <c r="C28" s="36" t="s">
         <v>53</v>
       </c>
       <c r="D28" s="33"/>
-      <c r="F28" s="37" t="s">
+      <c r="F28" s="36" t="s">
         <v>47</v>
       </c>
       <c r="G28" s="33"/>
-      <c r="H28" s="37" t="s">
+      <c r="H28" s="36" t="s">
         <v>54</v>
       </c>
       <c r="I28" s="33"/>
-      <c r="K28" s="37" t="s">
+      <c r="K28" s="36" t="s">
         <v>47</v>
       </c>
       <c r="L28" s="33"/>
-      <c r="M28" s="37" t="s">
+      <c r="M28" s="36" t="s">
         <v>55</v>
       </c>
       <c r="N28" s="33"/>
@@ -3955,19 +3957,19 @@
       <c r="A29" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="B29" s="36"/>
+      <c r="B29" s="35"/>
       <c r="C29" s="33"/>
       <c r="D29" s="33"/>
       <c r="F29" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="G29" s="36"/>
+      <c r="G29" s="35"/>
       <c r="H29" s="33"/>
       <c r="I29" s="33"/>
       <c r="K29" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="L29" s="36"/>
+      <c r="L29" s="35"/>
       <c r="M29" s="33"/>
       <c r="N29" s="33"/>
     </row>
@@ -3975,19 +3977,19 @@
       <c r="A30" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B30" s="35"/>
+      <c r="B30" s="34"/>
       <c r="C30" s="33"/>
       <c r="D30" s="33"/>
       <c r="F30" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="G30" s="35"/>
+      <c r="G30" s="34"/>
       <c r="H30" s="33"/>
       <c r="I30" s="33"/>
       <c r="K30" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="L30" s="35"/>
+      <c r="L30" s="34"/>
       <c r="M30" s="33"/>
       <c r="N30" s="33"/>
     </row>
@@ -3995,19 +3997,19 @@
       <c r="A31" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="B31" s="36"/>
+      <c r="B31" s="35"/>
       <c r="C31" s="33"/>
       <c r="D31" s="33"/>
       <c r="F31" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="G31" s="36"/>
+      <c r="G31" s="35"/>
       <c r="H31" s="33"/>
       <c r="I31" s="33"/>
       <c r="K31" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="L31" s="36"/>
+      <c r="L31" s="35"/>
       <c r="M31" s="33"/>
       <c r="N31" s="33"/>
     </row>
@@ -4015,19 +4017,19 @@
       <c r="A32" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B32" s="35"/>
+      <c r="B32" s="34"/>
       <c r="C32" s="33"/>
       <c r="D32" s="33"/>
       <c r="F32" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G32" s="35"/>
+      <c r="G32" s="34"/>
       <c r="H32" s="33"/>
       <c r="I32" s="33"/>
       <c r="K32" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="L32" s="35"/>
+      <c r="L32" s="34"/>
       <c r="M32" s="33"/>
       <c r="N32" s="33"/>
     </row>
@@ -4035,19 +4037,19 @@
       <c r="A33" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B33" s="36"/>
+      <c r="B33" s="35"/>
       <c r="C33" s="33"/>
       <c r="D33" s="33"/>
       <c r="F33" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="G33" s="36"/>
+      <c r="G33" s="35"/>
       <c r="H33" s="33"/>
       <c r="I33" s="33"/>
       <c r="K33" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="L33" s="36"/>
+      <c r="L33" s="35"/>
       <c r="M33" s="33"/>
       <c r="N33" s="33"/>
     </row>
@@ -4055,19 +4057,19 @@
       <c r="A34" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="B34" s="35"/>
+      <c r="B34" s="34"/>
       <c r="C34" s="33"/>
       <c r="D34" s="33"/>
       <c r="F34" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="G34" s="35"/>
+      <c r="G34" s="34"/>
       <c r="H34" s="33"/>
       <c r="I34" s="33"/>
       <c r="K34" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="L34" s="35"/>
+      <c r="L34" s="34"/>
       <c r="M34" s="33"/>
       <c r="N34" s="33"/>
     </row>
@@ -4075,19 +4077,19 @@
       <c r="A35" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="B35" s="36"/>
+      <c r="B35" s="35"/>
       <c r="C35" s="33"/>
       <c r="D35" s="33"/>
       <c r="F35" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="G35" s="36"/>
+      <c r="G35" s="35"/>
       <c r="H35" s="33"/>
       <c r="I35" s="33"/>
       <c r="K35" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="L35" s="36"/>
+      <c r="L35" s="35"/>
       <c r="M35" s="33"/>
       <c r="N35" s="33"/>
     </row>
@@ -4095,19 +4097,19 @@
       <c r="A36" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="B36" s="35"/>
+      <c r="B36" s="34"/>
       <c r="C36" s="33"/>
       <c r="D36" s="33"/>
       <c r="F36" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="G36" s="35"/>
+      <c r="G36" s="34"/>
       <c r="H36" s="33"/>
       <c r="I36" s="33"/>
       <c r="K36" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="L36" s="35"/>
+      <c r="L36" s="34"/>
       <c r="M36" s="33"/>
       <c r="N36" s="33"/>
     </row>
@@ -4115,7 +4117,7 @@
       <c r="A37" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="B37" s="38">
+      <c r="B37" s="37">
         <f>SUM(B29:B36)</f>
         <v>0</v>
       </c>
@@ -4124,7 +4126,7 @@
       <c r="F37" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="G37" s="38">
+      <c r="G37" s="37">
         <f>SUM(G29:G36)</f>
         <v>0</v>
       </c>
@@ -4133,7 +4135,7 @@
       <c r="K37" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="L37" s="38">
+      <c r="L37" s="37">
         <f>SUM(L29:L36)</f>
         <v>0</v>
       </c>
@@ -4170,6 +4172,68 @@
     </row>
   </sheetData>
   <mergeCells count="78">
+    <mergeCell ref="L34:N34"/>
+    <mergeCell ref="L6:N6"/>
+    <mergeCell ref="B33:D33"/>
+    <mergeCell ref="B32:D32"/>
+    <mergeCell ref="M28:N28"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="G11:I11"/>
+    <mergeCell ref="L7:N7"/>
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="L10:N10"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="L9:N9"/>
+    <mergeCell ref="F1:I1"/>
+    <mergeCell ref="L31:N31"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="F2:I2"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="K2:N2"/>
+    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="L5:N5"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="L37:N37"/>
+    <mergeCell ref="G8:I8"/>
+    <mergeCell ref="L12:N12"/>
+    <mergeCell ref="G10:I10"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="G34:I34"/>
+    <mergeCell ref="K25:N25"/>
+    <mergeCell ref="G29:I29"/>
+    <mergeCell ref="B35:D35"/>
+    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="G37:I37"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="L8:N8"/>
+    <mergeCell ref="G30:I30"/>
+    <mergeCell ref="G35:I35"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="L30:N30"/>
+    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="G33:I33"/>
+    <mergeCell ref="L29:N29"/>
+    <mergeCell ref="B31:D31"/>
+    <mergeCell ref="B6:D6"/>
+    <mergeCell ref="L11:N11"/>
+    <mergeCell ref="K26:N26"/>
+    <mergeCell ref="G9:I9"/>
+    <mergeCell ref="B5:D5"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="G13:I13"/>
+    <mergeCell ref="G12:I12"/>
+    <mergeCell ref="G5:I5"/>
     <mergeCell ref="G36:I36"/>
     <mergeCell ref="L32:N32"/>
     <mergeCell ref="L13:N13"/>
@@ -4186,68 +4250,6 @@
     <mergeCell ref="L33:N33"/>
     <mergeCell ref="L35:N35"/>
     <mergeCell ref="B34:D34"/>
-    <mergeCell ref="B6:D6"/>
-    <mergeCell ref="L11:N11"/>
-    <mergeCell ref="K26:N26"/>
-    <mergeCell ref="G9:I9"/>
-    <mergeCell ref="B5:D5"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="G5:I5"/>
-    <mergeCell ref="L30:N30"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="G33:I33"/>
-    <mergeCell ref="L29:N29"/>
-    <mergeCell ref="B31:D31"/>
-    <mergeCell ref="L37:N37"/>
-    <mergeCell ref="G8:I8"/>
-    <mergeCell ref="L12:N12"/>
-    <mergeCell ref="G10:I10"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="G34:I34"/>
-    <mergeCell ref="K25:N25"/>
-    <mergeCell ref="G29:I29"/>
-    <mergeCell ref="B35:D35"/>
-    <mergeCell ref="G31:I31"/>
-    <mergeCell ref="G37:I37"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="L8:N8"/>
-    <mergeCell ref="G30:I30"/>
-    <mergeCell ref="G35:I35"/>
-    <mergeCell ref="B37:D37"/>
-    <mergeCell ref="F1:I1"/>
-    <mergeCell ref="L31:N31"/>
-    <mergeCell ref="K4:L4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="F2:I2"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="K2:N2"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="L5:N5"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="K1:N1"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="L34:N34"/>
-    <mergeCell ref="L6:N6"/>
-    <mergeCell ref="B33:D33"/>
-    <mergeCell ref="B32:D32"/>
-    <mergeCell ref="M28:N28"/>
-    <mergeCell ref="A25:D25"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="G11:I11"/>
-    <mergeCell ref="L7:N7"/>
-    <mergeCell ref="F26:I26"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="L10:N10"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="L9:N9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>